<commit_message>
Point the matrix's Play URL at the new address; no redirect
The Settings sheet's Play URL is now
https://holytispoon.github.io/HEARsay-Mysteries/commons-comma/, and its
note says the build doesn't use it. Edited in the workbook's XML: only
xl/worksheets/sheet2.xml changed, and the rebuilt docs/ is unchanged.

ARCHITECTURE.md drops the plan to redirect the old Pages link.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KirxWu4F8J96Lg1LmBP2FD
</commit_message>
<xml_diff>
--- a/scenarios/commons-comma/The Commons' Comma – Response Matrix.xlsx
+++ b/scenarios/commons-comma/The Commons' Comma – Response Matrix.xlsx
@@ -2273,12 +2273,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>https://holytispoon.github.io/HEARsay-Mysteries-Commons-Comma/</t>
+          <t>https://holytispoon.github.io/HEARsay-Mysteries/commons-comma/</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>The GitHub Pages link, shown at the top of the repository README. Leave blank to omit.</t>
+          <t>The game's GitHub Pages link, for reference. The build doesn't use it.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Renumber the Clues C01–C16
The four dropped Clues left gaps; the remaining Clues are renumbered in order
(C06→C05 … C20→C16) in the matrix Sheet and the packet Doc, and copied here
from their downloads. Nothing else changed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scenarios/commons-comma/The Commons' Comma – Response Matrix.xlsx
+++ b/scenarios/commons-comma/The Commons' Comma – Response Matrix.xlsx
@@ -391,7 +391,7 @@
     <t>[R21 | unreceptive] Newsroom until ten to nine, comparing old scans, then out for air, then back. At 9:20 a courier dropped off a stiff, document-sized envelope and I signed for it. Who sent it is my business. Leo will tell you that's nothing. Leo would tell you a fire alarm was nothing if it interrupted a pitch.</t>
   </si>
   <si>
-    <t>[C13 | unreceptive] Catered the forum, then the café till close. About five to nine someone carried a long cardboard tube from the Commons toward the theatre; it had theatre paint on one end and nearly took out my sign. Couldn't see the face. Leo says I should have looked harder. Leo has never worked a counter.</t>
+    <t>[C10 | unreceptive] Catered the forum, then the café till close. About five to nine someone carried a long cardboard tube from the Commons toward the theatre; it had theatre paint on one end and nearly took out my sign. Couldn't see the face. Leo says I should have looked harder. Leo has never worked a counter.</t>
   </si>
   <si>
     <t>[R02 | receptive] I chaired the forum till 7:45, then the student-government office. On the way I saw Leo cross the Commons lobby, right by the archive corridor, at about 8:35. I don't think that means anything by itself; he was heading toward the business building. He and I disagree about nearly everything in the plan, and I still think he wants the same thing we all do, which is a building students use.</t>
@@ -400,7 +400,7 @@
     <t>Q2. Do you actually understand what the disputed comma changes, or should I explain it?</t>
   </si>
   <si>
-    <t>[C06 | receptive] I do understand it, though I appreciate you checking rather than assuming. I've argued for two years, in seminar and in the student paper, that the mark is an original comma, which makes students their own required approver. I may be wrong; my certainty isn't proof. Priya would say the same about her access logs, and she's right that a careful reading beats a confident one.</t>
+    <t>[C05 | receptive] I do understand it, though I appreciate you checking rather than assuming. I've argued for two years, in seminar and in the student paper, that the mark is an original comma, which makes students their own required approver. I may be wrong; my certainty isn't proof. Priya would say the same about her access logs, and she's right that a careful reading beats a confident one.</t>
   </si>
   <si>
     <t>[R05 | unreceptive] Obviously I understand it. Comma, no comma, students get a veto or they don't. The people who really understand the mechanics are the tech kids; Priya had the access dashboard open on her second monitor all evening, so if anyone could have touched a log, it's her. Mira thinks a two-year seminar makes her an expert on ink. It makes her an expert on delay.</t>
@@ -409,19 +409,19 @@
     <t>TW — Priya's face goes flat. “I wrote the explainer. If you need the comma explained to me, we're finished.” She turns back to her screen.</t>
   </si>
   <si>
-    <t>[C17 | receptive] I understand it well enough to know why Mira cares. We argue about whether the theatre should block the whole plan, and we probably always will, but on one thing we're the same: the Charter should not get damaged or lost. I might be naïve about the politics. I'm not naïve about paper in a damp building.</t>
+    <t>[C14 | receptive] I understand it well enough to know why Mira cares. We argue about whether the theatre should block the whole plan, and we probably always will, but on one thing we're the same: the Charter should not get damaged or lost. I might be naïve about the politics. I'm not naïve about paper in a damp building.</t>
   </si>
   <si>
     <t>[R24 | receptive] I think I do, though Mira understands it better. I've heard the rumour that someone meant to settle it last night with a chemistry test on the ink. That couldn't happen: dating ink needs a sample scraped from the document and about a week of lab work, and I checked for the audit that every chemistry-building door locks at six on event nights. I can't judge the comma myself. Priya would want the timestamps first, and I think that's the sensible order.</t>
   </si>
   <si>
-    <t>[C07 | receptive] I understand it, and I'd rather be corrected than assumed to. What I can say is this: in the photograph we printed, the disputed mark has sharper edges and a different paper shadow than the surrounding ink. Mira noticed it before I did. I may be wrong about what it means; she and I disagree about whether the examination should go ahead at all, and she's right that a careful result would help everyone.</t>
+    <t>[C06 | receptive] I understand it, and I'd rather be corrected than assumed to. What I can say is this: in the photograph we printed, the disputed mark has sharper edges and a different paper shadow than the surrounding ink. Mira noticed it before I did. I may be wrong about what it means; she and I disagree about whether the examination should go ahead at all, and she's right that a careful result would help everyone.</t>
   </si>
   <si>
     <t>[R16 | unreceptive] I don't and I don't need to. I delivered coffee to the meeting room where they were arguing about it at 7:20, and Hana was signing in to get a folder while the forum was still going. Mira can explain the comma to you for an hour. It won't make the café stay open.</t>
   </si>
   <si>
-    <t>[C06 | receptive] I think so, though Mira would explain it better. She's argued for months that the mark is an original comma, which would give students their own required approval. I try to hold that lightly; a lot of us want it to be a comma, and wanting it isn't evidence. Leo says the whole debate is delay. He has a point about the delay, even if I don't agree about the debate.</t>
+    <t>[C05 | receptive] I think so, though Mira would explain it better. She's argued for months that the mark is an original comma, which would give students their own required approval. I try to hold that lightly; a lot of us want it to be a comma, and wanting it isn't evidence. Leo says the whole debate is delay. He has a point about the delay, even if I don't agree about the debate.</t>
   </si>
   <si>
     <t>Q3. Who have you been talking to about the Charter, and what did they tell you?</t>
@@ -433,19 +433,19 @@
     <t>[C04 | unreceptive] Ellison, mostly, about the invitations. He told me nobody except Mira Shah's credential opened the archive between the forum and closing. That should settle it, but it won't, because Sofia will find a way to make one card swipe into a conspiracy. She's not a journalist, she's an activist with a byline.</t>
   </si>
   <si>
-    <t>[C08 | receptive] Mira, a few days ago. She asked me to compare the newspaper photograph with older images of the Charter. I might be wrong about what it means, but a small crease near the mark that shows in the older photographs isn't in the newspaper one. Mira and I don't agree about facial recognition, and I still think she's right that images deserve the same scrutiny as logs.</t>
-  </si>
-  <si>
-    <t>[C12 | unreceptive] Mira, last night. She needed a container and I gave her an empty poster tube, the one labelled 'Spring Gala 2023'. That's it. Now Sofia is sniffing around the loft as if a cardboard tube proves a conspiracy. She wants a scandal more than she wants an answer.</t>
-  </si>
-  <si>
-    <t>[C09 | receptive] Students at the forum, and one administrator: Celia Park kept asking how the university would describe the result, and pressing for 'a clean answer' for the Board. Around the same time the event materials stopped saying 'the original Charter' and just said 'the Charter'. That may be ordinary legal caution, as Leo says; he's probably right that it isn't proof of anything by itself.</t>
+    <t>[C07 | receptive] Mira, a few days ago. She asked me to compare the newspaper photograph with older images of the Charter. I might be wrong about what it means, but a small crease near the mark that shows in the older photographs isn't in the newspaper one. Mira and I don't agree about facial recognition, and I still think she's right that images deserve the same scrutiny as logs.</t>
+  </si>
+  <si>
+    <t>[C09 | unreceptive] Mira, last night. She needed a container and I gave her an empty poster tube, the one labelled 'Spring Gala 2023'. That's it. Now Sofia is sniffing around the loft as if a cardboard tube proves a conspiracy. She wants a scandal more than she wants an answer.</t>
+  </si>
+  <si>
+    <t>[C08 | receptive] Students at the forum, and one administrator: Celia Park kept asking how the university would describe the result, and pressing for 'a clean answer' for the Board. Around the same time the event materials stopped saying 'the original Charter' and just said 'the Charter'. That may be ordinary legal caution, as Leo says; he's probably right that it isn't proof of anything by itself.</t>
   </si>
   <si>
     <t>TW — Sofia's tone drops. “I don't name sources. Not for the president, not for you.” She picks up her bag and goes.</t>
   </si>
   <si>
-    <t>[C20 | receptive] Mira, at the counter, around ten to nine. She said she'd 'keep it safe until someone can compare the two'. I didn't ask what 'it' was. Maybe I should have; Sofia would have. She and I want different things from all this, but she's right that people say important things to whoever's pouring the tea.</t>
+    <t>[C16 | receptive] Mira, at the counter, around ten to nine. She said she'd 'keep it safe until someone can compare the two'. I didn't ask what 'it' was. Maybe I should have; Sofia would have. She and I want different things from all this, but she's right that people say important things to whoever's pouring the tea.</t>
   </si>
   <si>
     <t>[R22 | receptive] Sofia, and I should own something before it comes out another way: I gave her the draft resolution that ran this morning. That was my call, and probably a mistake. She showed me the envelope she signed for last night; it was the printer's proof of today's front page, and it's pinned on the newsroom wall. Sofia thinks worries like mine are a story. She may be right that it's worth checking; I'd just want to check with people, not around them.</t>
@@ -457,7 +457,7 @@
     <t>[R19 | receptive] It could be, but not the way you might think. The theatre does have a 'Commons Charter': a printed prop from the 2019 Founders' Day play, on modern paper and a third smaller than the real one. It was signed out for a costume fitting last week, and anyone who has handled the original would know the difference across a room. Jonah and I disagree about whether the theatre should block the whole plan, and I think he's right that the loft is one of the few places on campus that's actually dry and dark.</t>
   </si>
   <si>
-    <t>[C13 | unreceptive] Probably. Around five to nine I saw someone hauling a long cardboard tube from the Commons toward the theatre; it had paint on one end, the way all Jonah's tubes do. Theatre people carry tubes constantly, which is exactly why nobody looks. Jonah will tell you the loft is sacred. It's a fire hazard with a curtain.</t>
+    <t>[C10 | unreceptive] Probably. Around five to nine I saw someone hauling a long cardboard tube from the Commons toward the theatre; it had paint on one end, the way all Jonah's tubes do. Theatre people carry tubes constantly, which is exactly why nobody looks. Jonah will tell you the loft is sacred. It's a fire hazard with a curtain.</t>
   </si>
   <si>
     <t>[R18 | unreceptive] Check the equipment-booking system before you check the gossip. It shows the theatre signed out an item called 'Commons Charter' last week, and it hasn't come back. That's a record, not a rumour. Jonah acts like the loft is off-limits to questions. It's a room.</t>
@@ -466,25 +466,25 @@
     <t>TW — Jonah sets down the cable coil. “So the theatre is your suspect. If you have evidence, show it. If not, stay out of my loft.” He walks away.</t>
   </si>
   <si>
-    <t>[C15 | receptive] It could be; the loft is dry, which is more than most of the building. I was there for the accessibility audit and noticed tubes had been moved and the inventory sheet didn't match. Jonah would say the loft isn't a public room, and he's right; I'd only add that good storage and good access turn out to be the same problem, which is something he and I agree on.</t>
-  </si>
-  <si>
-    <t>[C14 | unreceptive] Jonah told me a poster tube in the loft had got heavier since last night. I asked him not to move it again. He treats the loft like a chapel, which is charming and useless. If he'd run an inventory like a normal person we wouldn't be guessing.</t>
+    <t>[C12 | receptive] It could be; the loft is dry, which is more than most of the building. I was there for the accessibility audit and noticed tubes had been moved and the inventory sheet didn't match. Jonah would say the loft isn't a public room, and he's right; I'd only add that good storage and good access turn out to be the same problem, which is something he and I agree on.</t>
+  </si>
+  <si>
+    <t>[C11 | unreceptive] Jonah told me a poster tube in the loft had got heavier since last night. I asked him not to move it again. He treats the loft like a chapel, which is charming and useless. If he'd run an inventory like a normal person we wouldn't be guessing.</t>
   </si>
   <si>
     <t>[R17 | unreceptive] Could be. When I locked up I saw a rolled parchment that looked just like the Charter lying on the costume trunk by the stage door. Didn't touch it. Jonah thinks the loft is the last honest room on campus. It's a loft with a leak on the north side.</t>
   </si>
   <si>
-    <t>[C12 | receptive] Possibly. I saw Jonah hand Mira a poster tube near the theatre; I could read 'Spring Gala' on the label. I assumed it was for scenery paperwork, and it may have been. Jonah would say the theatre gets blamed for everything, and I can see why he feels that; it's also probably why he'd be the person you'd ask for a safe place to keep something.</t>
+    <t>[C09 | receptive] Possibly. I saw Jonah hand Mira a poster tube near the theatre; I could read 'Spring Gala' on the label. I assumed it was for scenery paperwork, and it may have been. Jonah would say the theatre gets blamed for everything, and I can see why he feels that; it's also probably why he'd be the person you'd ask for a safe place to keep something.</t>
   </si>
   <si>
     <t>Q5. Isn't the missing Charter just a political football at this point?</t>
   </si>
   <si>
-    <t>[C19 | unreceptive] No. Calling it a football is what people say when they'd rather not look at the evidence. The steering group doesn't even hold archive credentials; they go through the archivist's office, and nobody used that route last night. Hana treats every administrative shortcut as a conspiracy. This one isn't; it's just procedure.</t>
-  </si>
-  <si>
-    <t>[C09 | unreceptive] It's been a football since the forum. The event materials changed late; first it was an examination of 'the original Charter', then just 'the Charter', because Celia Park wanted a clean answer for the Board. That's communications people being communications people. Hana reads it as a plot. Hana reads everything as a plot.</t>
+    <t>[C15 | unreceptive] No. Calling it a football is what people say when they'd rather not look at the evidence. The steering group doesn't even hold archive credentials; they go through the archivist's office, and nobody used that route last night. Hana treats every administrative shortcut as a conspiracy. This one isn't; it's just procedure.</t>
+  </si>
+  <si>
+    <t>[C08 | unreceptive] It's been a football since the forum. The event materials changed late; first it was an examination of 'the original Charter', then just 'the Charter', because Celia Park wanted a clean answer for the Board. That's communications people being communications people. Hana reads it as a plot. Hana reads everything as a plot.</t>
   </si>
   <si>
     <t>[R03 | unreceptive] It's an evidence question, not a political one. While people are pointing at Leo, the incubator badge reader has him in the business building from 8:36 until after 9:10. He couldn't have been in the archive at 8:42 or at a terminal at 9:17. Sofia would rather run the rumour than the log. That's the difference between us.</t>
@@ -508,7 +508,7 @@
     <t>Q6. Does any of this actually matter to you?</t>
   </si>
   <si>
-    <t>[C07 | receptive] It matters more than anything I've worked on. When I saw the newspaper photograph, the disputed mark had sharper edges and a different paper shadow than the ink around it. I could be reading too much into a printed image, and I understand why the renovation supporters want the examination to go ahead. So do I. I just want the object on the table to be the real one.</t>
+    <t>[C06 | receptive] It matters more than anything I've worked on. When I saw the newspaper photograph, the disputed mark had sharper edges and a different paper shadow than the ink around it. I could be reading too much into a printed image, and I understand why the renovation supporters want the examination to go ahead. So do I. I just want the object on the table to be the real one.</t>
   </si>
   <si>
     <t>[R01 | unreceptive] Yes, and I'll save you the discovery: the committee told me the club would get first choice of new office space. That makes my support look bought. It isn't. I wanted the building before anyone offered me anything, and no amount of Nia's compromise talk changes the fact that the current Commons is a museum with bad Wi-Fi.</t>
@@ -517,7 +517,7 @@
     <t>[C04 | receptive] It matters, though maybe not in the way you'd expect. I care that the system is read correctly: no credential other than Mira's opened the archive between the forum and closing. That doesn't tell you what she did inside, and I'd want to hear her account before drawing a line from a swipe to a theft. Hana's right that a log records entry, not intent.</t>
   </si>
   <si>
-    <t>[C14 | receptive] It matters. That 'Spring Gala 2023' tube is up in the scenery loft now, and it's heavier than an empty tube has any business being. I haven't opened it. I should probably admit that Priya's point about chains of custody applies to my loft as much as to her logs, and that I'd feel better if someone from the archive looked before anyone else does.</t>
+    <t>[C11 | receptive] It matters. That 'Spring Gala 2023' tube is up in the scenery loft now, and it's heavier than an empty tube has any business being. I haven't opened it. I should probably admit that Priya's point about chains of custody applies to my loft as much as to her logs, and that I'd feel better if someone from the archive looked before anyone else does.</t>
   </si>
   <si>
     <t>[R09 | receptive] It does, though maybe less than the café does to Evan, and that's fine. Since you'll hear about it: the tube in Evan's locker held catering menus and inventory sheets, and it was there before the forum ended. He and I want different things from this building and we both want people treated decently in it.</t>
@@ -529,7 +529,7 @@
     <t>TW — Evan stops wiping the counter. “You want my observations, then tell me they don't count. Pick one.” He goes into the back.</t>
   </si>
   <si>
-    <t>[C20 | receptive] It matters to me because I promised the forum a fair process. Mira told me she'd keep something safe 'until someone can compare the two'. I'm fairly sure she meant to give it back. I know Sofia would say that's naïve, and she's often right about the administration; I'd like to be right about a person for once.</t>
+    <t>[C16 | receptive] It matters to me because I promised the forum a fair process. Mira told me she'd keep something safe 'until someone can compare the two'. I'm fairly sure she meant to give it back. I know Sofia would say that's naïve, and she's often right about the administration; I'd like to be right about a person for once.</t>
   </si>
   <si>
     <t>Q7. Whose side are you really on?</t>
@@ -547,13 +547,13 @@
     <t>[R07 | unreceptive] The theatre's. Since you're asking whose side, ask the café. Evan had a document tube sitting in his locker overnight. Nobody's interrogating him, because Evan says he doesn't care and everyone believes him. Leo would say that's proof the theatre's a distraction. Leo would say anything that ends the conversation.</t>
   </si>
   <si>
-    <t>[C17 | receptive] On the side of a building that lets everyone in. Mira and Jonah are on different sides of the theatre question and I've watched them argue about it, but they agree the Charter must not be damaged or lost. I think that's worth more than either of them realizes, and it's probably why they trust each other.</t>
+    <t>[C14 | receptive] On the side of a building that lets everyone in. Mira and Jonah are on different sides of the theatre question and I've watched them argue about it, but they agree the Charter must not be damaged or lost. I think that's worth more than either of them realizes, and it's probably why they trust each other.</t>
   </si>
   <si>
     <t>[R10 | unreceptive] The public's. Which is why I'll tell you Martin Ellison, the archivist, was hanging around the archive office at half past eight. Nobody in the administration will explain what he was doing. Evan says he saw nothing unusual. Evan wouldn't notice a fire unless it was in the espresso machine.</t>
   </si>
   <si>
-    <t>[C16 | receptive] Nobody's. Since you ask fairly: around ten to nine I saw Mira and Jonah talking by the theatre. It looked like two people sorting out where to put something, not an argument. I could be wrong; I was fifty feet away. Nia says everyone in this is on the same side underneath. That's more generous than I'd be, but she might be right.</t>
+    <t>[C13 | receptive] Nobody's. Since you ask fairly: around ten to nine I saw Mira and Jonah talking by the theatre. It looked like two people sorting out where to put something, not an argument. I could be wrong; I was fifty feet away. Nia says everyone in this is on the same side underneath. That's more generous than I'd be, but she might be right.</t>
   </si>
   <si>
     <t>TW — Nia flushes. “I'm not answering a loyalty test. I told you what I think.” She ends the conversation.</t>
@@ -571,19 +571,19 @@
     <t>[R04 | unreceptive] No. I copied a debugging file from the access system without permission, and I regret it, and it's going to come out anyway. It has credential events in it, nothing else. Leo will call it a distraction. Leo calls anything he doesn't understand a distraction.</t>
   </si>
   <si>
-    <t>[C15 | receptive] No, and I'll tell you the thing that makes me look bad: after Mira left I moved several tubes around in the loft to keep rain off the paper stock and never updated the inventory. That's sloppy, not sinister. Hana's told me for a year that bad storage and bad access are the same institutional problem. She's right, and I should have listened sooner.</t>
-  </si>
-  <si>
-    <t>[C19 | receptive] No. I've checked the other obvious suspicion for you, since it's the one Sofia keeps raising: steering-group members don't hold archive credentials at all. They reach the archive through the archivist's office, and nobody used that route last night. Sofia may still be right about their motives; she's just wrong about their access.</t>
-  </si>
-  <si>
-    <t>[C08 | unreceptive] No. I have something better: there's a small crease near the mark in the older photographs of the Charter. It isn't in the photo we printed of the examination copy. Mira flagged it. Priya says an image needs the same care as a log. Fine. The image says what it says.</t>
+    <t>[C12 | receptive] No, and I'll tell you the thing that makes me look bad: after Mira left I moved several tubes around in the loft to keep rain off the paper stock and never updated the inventory. That's sloppy, not sinister. Hana's told me for a year that bad storage and bad access are the same institutional problem. She's right, and I should have listened sooner.</t>
+  </si>
+  <si>
+    <t>[C15 | receptive] No. I've checked the other obvious suspicion for you, since it's the one Sofia keeps raising: steering-group members don't hold archive credentials at all. They reach the archive through the archivist's office, and nobody used that route last night. Sofia may still be right about their motives; she's just wrong about their access.</t>
+  </si>
+  <si>
+    <t>[C07 | unreceptive] No. I have something better: there's a small crease near the mark in the older photographs of the Charter. It isn't in the photo we printed of the examination copy. Mira flagged it. Priya says an image needs the same care as a log. Fine. The image says what it says.</t>
   </si>
   <si>
     <t>[R08 | unreceptive] No. I let somebody I didn't recognize use my locker around half past eight because it was raining and I wanted to get back to work. That's careless, not criminal. Sofia will make it a headline anyway. Sofia would make the rain a headline.</t>
   </si>
   <si>
-    <t>[C16 | receptive] No. What I can tell you is that I saw Mira and Jonah talking near the theatre at about ten to nine, and it looked like a practical conversation about where to put something, not a confrontation. I might be misreading it from a distance. Leo would read it as proof. I'd rather ask them; both of them want the Charter kept safe, which is more than the two sides of this fight usually share.</t>
+    <t>[C13 | receptive] No. What I can tell you is that I saw Mira and Jonah talking near the theatre at about ten to nine, and it looked like a practical conversation about where to put something, not a confrontation. I might be misreading it from a distance. Leo would read it as proof. I'd rather ask them; both of them want the Charter kept safe, which is more than the two sides of this fight usually share.</t>
   </si>
   <si>
     <t>Witness ID</t>
@@ -637,372 +637,372 @@
     <t>Do you actually understand what the disputed comma changes, or should I explain it?</t>
   </si>
   <si>
+    <t>C05</t>
+  </si>
+  <si>
+    <t>MC2</t>
+  </si>
+  <si>
+    <t>I do understand it, though I appreciate you checking rather than assuming. I've argued for two years, in seminar and in the student paper, that the mark is an original comma, which makes students their own required approver. I may be wrong; my certainty isn't proof. Priya would say the same about her access logs, and she's right that a careful reading beats a confident one.</t>
+  </si>
+  <si>
+    <t>Q3</t>
+  </si>
+  <si>
+    <t>Who have you been talking to about the Charter, and what did they tell you?</t>
+  </si>
+  <si>
+    <t>R13</t>
+  </si>
+  <si>
+    <t>red herring</t>
+  </si>
+  <si>
+    <t>S5</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>Sofia, mostly. She was in the newsroom late comparing old scans, and she's the one who printed the photograph. You should know she once ran a detail she hadn't verified. Anyone who reads her coverage as neutral is kidding themselves. She's decided the administration is corrupt and she's looking for facts to fit.</t>
+  </si>
+  <si>
+    <t>Q4</t>
+  </si>
+  <si>
+    <t>Could the Charter be hidden somewhere in the theatre?</t>
+  </si>
+  <si>
+    <t>R19</t>
+  </si>
+  <si>
+    <t>S7</t>
+  </si>
+  <si>
+    <t>It could be, but not the way you might think. The theatre does have a 'Commons Charter': a printed prop from the 2019 Founders' Day play, on modern paper and a third smaller than the real one. It was signed out for a costume fitting last week, and anyone who has handled the original would know the difference across a room. Jonah and I disagree about whether the theatre should block the whole plan, and I think he's right that the loft is one of the few places on campus that's actually dry and dark.</t>
+  </si>
+  <si>
+    <t>Q5</t>
+  </si>
+  <si>
+    <t>Isn't the missing Charter just a political football at this point?</t>
+  </si>
+  <si>
+    <t>C15</t>
+  </si>
+  <si>
+    <t>MC4</t>
+  </si>
+  <si>
+    <t>No. Calling it a football is what people say when they'd rather not look at the evidence. The steering group doesn't even hold archive credentials; they go through the archivist's office, and nobody used that route last night. Hana treats every administrative shortcut as a conspiracy. This one isn't; it's just procedure.</t>
+  </si>
+  <si>
+    <t>Q6</t>
+  </si>
+  <si>
+    <t>Does any of this actually matter to you?</t>
+  </si>
+  <si>
     <t>C06</t>
   </si>
   <si>
-    <t>MC2</t>
-  </si>
-  <si>
-    <t>I do understand it, though I appreciate you checking rather than assuming. I've argued for two years, in seminar and in the student paper, that the mark is an original comma, which makes students their own required approver. I may be wrong; my certainty isn't proof. Priya would say the same about her access logs, and she's right that a careful reading beats a confident one.</t>
-  </si>
-  <si>
-    <t>Q3</t>
-  </si>
-  <si>
-    <t>Who have you been talking to about the Charter, and what did they tell you?</t>
-  </si>
-  <si>
-    <t>R13</t>
-  </si>
-  <si>
-    <t>red herring</t>
-  </si>
-  <si>
-    <t>S5</t>
-  </si>
-  <si>
-    <t>no</t>
-  </si>
-  <si>
-    <t>Sofia, mostly. She was in the newsroom late comparing old scans, and she's the one who printed the photograph. You should know she once ran a detail she hadn't verified. Anyone who reads her coverage as neutral is kidding themselves. She's decided the administration is corrupt and she's looking for facts to fit.</t>
-  </si>
-  <si>
-    <t>Q4</t>
-  </si>
-  <si>
-    <t>Could the Charter be hidden somewhere in the theatre?</t>
-  </si>
-  <si>
-    <t>R19</t>
-  </si>
-  <si>
-    <t>S7</t>
-  </si>
-  <si>
-    <t>It could be, but not the way you might think. The theatre does have a 'Commons Charter': a printed prop from the 2019 Founders' Day play, on modern paper and a third smaller than the real one. It was signed out for a costume fitting last week, and anyone who has handled the original would know the difference across a room. Jonah and I disagree about whether the theatre should block the whole plan, and I think he's right that the loft is one of the few places on campus that's actually dry and dark.</t>
-  </si>
-  <si>
-    <t>Q5</t>
-  </si>
-  <si>
-    <t>Isn't the missing Charter just a political football at this point?</t>
-  </si>
-  <si>
-    <t>C19</t>
-  </si>
-  <si>
-    <t>MC4</t>
-  </si>
-  <si>
-    <t>No. Calling it a football is what people say when they'd rather not look at the evidence. The steering group doesn't even hold archive credentials; they go through the archivist's office, and nobody used that route last night. Hana treats every administrative shortcut as a conspiracy. This one isn't; it's just procedure.</t>
-  </si>
-  <si>
-    <t>Q6</t>
-  </si>
-  <si>
-    <t>Does any of this actually matter to you?</t>
+    <t>It matters more than anything I've worked on. When I saw the newspaper photograph, the disputed mark had sharper edges and a different paper shadow than the ink around it. I could be reading too much into a printed image, and I understand why the renovation supporters want the examination to go ahead. So do I. I just want the object on the table to be the real one.</t>
+  </si>
+  <si>
+    <t>Q7</t>
+  </si>
+  <si>
+    <t>Whose side are you really on?</t>
+  </si>
+  <si>
+    <t>R06</t>
+  </si>
+  <si>
+    <t>S2</t>
+  </si>
+  <si>
+    <t>On the side of the document. People are whispering about Priya because she copied a file from the access system. I've read the archive's rules: that file only holds credential events, and editing the log needs an archive credential she doesn't have. She and I disagree about facial recognition, but she's right that we should separate what the system shows from what we fear it shows.</t>
+  </si>
+  <si>
+    <t>Q8</t>
+  </si>
+  <si>
+    <t>Did you remove the Charter, or touch the access log?</t>
+  </si>
+  <si>
+    <t>TRIPWIRE</t>
+  </si>
+  <si>
+    <t>tripwire</t>
+  </si>
+  <si>
+    <t>Mira's expression hardens. “If you have already decided what I did, there is no point in asking me anything.” She gathers her papers and leaves.</t>
+  </si>
+  <si>
+    <t>W02</t>
+  </si>
+  <si>
+    <t>Leo doesn't look up from his phone. “Minute by minute? I have a pitch review in ten minutes. Ask someone with time to spare.” He's gone.</t>
+  </si>
+  <si>
+    <t>R05</t>
+  </si>
+  <si>
+    <t>Obviously I understand it. Comma, no comma, students get a veto or they don't. The people who really understand the mechanics are the tech kids; Priya had the access dashboard open on her second monitor all evening, so if anyone could have touched a log, it's her. Mira thinks a two-year seminar makes her an expert on ink. It makes her an expert on delay.</t>
+  </si>
+  <si>
+    <t>C04</t>
+  </si>
+  <si>
+    <t>Ellison, mostly, about the invitations. He told me nobody except Mira Shah's credential opened the archive between the forum and closing. That should settle it, but it won't, because Sofia will find a way to make one card swipe into a conspiracy. She's not a journalist, she's an activist with a byline.</t>
+  </si>
+  <si>
+    <t>C10</t>
+  </si>
+  <si>
+    <t>MC3</t>
+  </si>
+  <si>
+    <t>Probably. Around five to nine I saw someone hauling a long cardboard tube from the Commons toward the theatre; it had paint on one end, the way all Jonah's tubes do. Theatre people carry tubes constantly, which is exactly why nobody looks. Jonah will tell you the loft is sacred. It's a fire hazard with a curtain.</t>
+  </si>
+  <si>
+    <t>C08</t>
+  </si>
+  <si>
+    <t>It's been a football since the forum. The event materials changed late; first it was an examination of 'the original Charter', then just 'the Charter', because Celia Park wanted a clean answer for the Board. That's communications people being communications people. Hana reads it as a plot. Hana reads everything as a plot.</t>
+  </si>
+  <si>
+    <t>R01</t>
+  </si>
+  <si>
+    <t>S1</t>
+  </si>
+  <si>
+    <t>Yes, and I'll save you the discovery: the committee told me the club would get first choice of new office space. That makes my support look bought. It isn't. I wanted the building before anyone offered me anything, and no amount of Nia's compromise talk changes the fact that the current Commons is a museum with bad Wi-Fi.</t>
+  </si>
+  <si>
+    <t>R20</t>
+  </si>
+  <si>
+    <t>S8</t>
+  </si>
+  <si>
+    <t>On the side of getting things built. If you want to know whose side people are on, ask who's feeding Sofia's paper: a draft student-government resolution that only a handful of people had was in this morning's edition. Somebody is passing her documents. I'm not going to pretend, like Nia does, that everyone in this is acting in good faith.</t>
+  </si>
+  <si>
+    <t>C01</t>
+  </si>
+  <si>
+    <t>No. I last saw the Charter at the forum at 7:45, in a blue archival folder, seal intact, before it went back to the cabinet. I didn't touch it. Anyone who thinks I'd risk the Board's whole process to steal a document I want examined hasn't thought about it for five seconds. Sofia hasn't.</t>
+  </si>
+  <si>
+    <t>W03</t>
+  </si>
+  <si>
+    <t>C03</t>
+  </si>
+  <si>
+    <t>I was in the lab until about 8:55 with the access dashboard open. The thing worth your time is this: the archive log was edited at 9:17 p.m., after the archive closed at nine, and edits need an archive credential, not maintenance or admin. Leo thinks logs are trivia. That's because he's never read one.</t>
+  </si>
+  <si>
+    <t>Priya's face goes flat. “I wrote the explainer. If you need the comma explained to me, we're finished.” She turns back to her screen.</t>
   </si>
   <si>
     <t>C07</t>
   </si>
   <si>
-    <t>It matters more than anything I've worked on. When I saw the newspaper photograph, the disputed mark had sharper edges and a different paper shadow than the ink around it. I could be reading too much into a printed image, and I understand why the renovation supporters want the examination to go ahead. So do I. I just want the object on the table to be the real one.</t>
-  </si>
-  <si>
-    <t>Q7</t>
-  </si>
-  <si>
-    <t>Whose side are you really on?</t>
-  </si>
-  <si>
-    <t>R06</t>
-  </si>
-  <si>
-    <t>S2</t>
-  </si>
-  <si>
-    <t>On the side of the document. People are whispering about Priya because she copied a file from the access system. I've read the archive's rules: that file only holds credential events, and editing the log needs an archive credential she doesn't have. She and I disagree about facial recognition, but she's right that we should separate what the system shows from what we fear it shows.</t>
-  </si>
-  <si>
-    <t>Q8</t>
-  </si>
-  <si>
-    <t>Did you remove the Charter, or touch the access log?</t>
-  </si>
-  <si>
-    <t>TRIPWIRE</t>
-  </si>
-  <si>
-    <t>tripwire</t>
-  </si>
-  <si>
-    <t>Mira's expression hardens. “If you have already decided what I did, there is no point in asking me anything.” She gathers her papers and leaves.</t>
-  </si>
-  <si>
-    <t>W02</t>
-  </si>
-  <si>
-    <t>Leo doesn't look up from his phone. “Minute by minute? I have a pitch review in ten minutes. Ask someone with time to spare.” He's gone.</t>
-  </si>
-  <si>
-    <t>R05</t>
-  </si>
-  <si>
-    <t>Obviously I understand it. Comma, no comma, students get a veto or they don't. The people who really understand the mechanics are the tech kids; Priya had the access dashboard open on her second monitor all evening, so if anyone could have touched a log, it's her. Mira thinks a two-year seminar makes her an expert on ink. It makes her an expert on delay.</t>
-  </si>
-  <si>
-    <t>C04</t>
-  </si>
-  <si>
-    <t>Ellison, mostly, about the invitations. He told me nobody except Mira Shah's credential opened the archive between the forum and closing. That should settle it, but it won't, because Sofia will find a way to make one card swipe into a conspiracy. She's not a journalist, she's an activist with a byline.</t>
+    <t>Mira, a few days ago. She asked me to compare the newspaper photograph with older images of the Charter. I might be wrong about what it means, but a small crease near the mark that shows in the older photographs isn't in the newspaper one. Mira and I don't agree about facial recognition, and I still think she's right that images deserve the same scrutiny as logs.</t>
+  </si>
+  <si>
+    <t>R18</t>
+  </si>
+  <si>
+    <t>Check the equipment-booking system before you check the gossip. It shows the theatre signed out an item called 'Commons Charter' last week, and it hasn't come back. That's a record, not a rumour. Jonah acts like the loft is off-limits to questions. It's a room.</t>
+  </si>
+  <si>
+    <t>R03</t>
+  </si>
+  <si>
+    <t>It's an evidence question, not a political one. While people are pointing at Leo, the incubator badge reader has him in the business building from 8:36 until after 9:10. He couldn't have been in the archive at 8:42 or at a terminal at 9:17. Sofia would rather run the rumour than the log. That's the difference between us.</t>
+  </si>
+  <si>
+    <t>It matters, though maybe not in the way you'd expect. I care that the system is read correctly: no credential other than Mira's opened the archive between the forum and closing. That doesn't tell you what she did inside, and I'd want to hear her account before drawing a line from a swipe to a theft. Hana's right that a log records entry, not intent.</t>
+  </si>
+  <si>
+    <t>On the side of what the record shows. Mira's credential opened the archive at 8:42; an ordinary entry, no forced door. I know Leo reads that as case closed, and he may turn out to be right. I'd just rather we got there by asking what an ordinary entry means when the person has every right to be there.</t>
+  </si>
+  <si>
+    <t>R04</t>
+  </si>
+  <si>
+    <t>No. I copied a debugging file from the access system without permission, and I regret it, and it's going to come out anyway. It has credential events in it, nothing else. Leo will call it a distraction. Leo calls anything he doesn't understand a distraction.</t>
+  </si>
+  <si>
+    <t>W04</t>
+  </si>
+  <si>
+    <t>R23</t>
+  </si>
+  <si>
+    <t>S9</t>
+  </si>
+  <si>
+    <t>Loading dock from half past seven to nearly nine, wrangling a lighting case. Around twenty to nine Evan slipped out of the café for ten minutes and came back from the direction of the chemistry building, and somebody at the forum had joked that the comma's ink could be tested in a lab tonight. I didn't ask him about it. Leo would say I should have. He might be right; theatre people are so used to things moving that we stop asking.</t>
+  </si>
+  <si>
+    <t>C14</t>
+  </si>
+  <si>
+    <t>I understand it well enough to know why Mira cares. We argue about whether the theatre should block the whole plan, and we probably always will, but on one thing we're the same: the Charter should not get damaged or lost. I might be naïve about the politics. I'm not naïve about paper in a damp building.</t>
+  </si>
+  <si>
+    <t>C09</t>
+  </si>
+  <si>
+    <t>Mira, last night. She needed a container and I gave her an empty poster tube, the one labelled 'Spring Gala 2023'. That's it. Now Sofia is sniffing around the loft as if a cardboard tube proves a conspiracy. She wants a scandal more than she wants an answer.</t>
+  </si>
+  <si>
+    <t>Jonah sets down the cable coil. “So the theatre is your suspect. If you have evidence, show it. If not, stay out of my loft.” He walks away.</t>
+  </si>
+  <si>
+    <t>R15</t>
+  </si>
+  <si>
+    <t>S6</t>
+  </si>
+  <si>
+    <t>Everything is a football to the people kicking it. Want something concrete? Hana went into the steering group's restricted meeting room. I saw her come out with a folder. She'll tell you it was for accessibility. Maybe. She also never misses a chance to make the administration look bad.</t>
+  </si>
+  <si>
+    <t>C11</t>
+  </si>
+  <si>
+    <t>It matters. That 'Spring Gala 2023' tube is up in the scenery loft now, and it's heavier than an empty tube has any business being. I haven't opened it. I should probably admit that Priya's point about chains of custody applies to my loft as much as to her logs, and that I'd feel better if someone from the archive looked before anyone else does.</t>
+  </si>
+  <si>
+    <t>R07</t>
+  </si>
+  <si>
+    <t>S3</t>
+  </si>
+  <si>
+    <t>The theatre's. Since you're asking whose side, ask the café. Evan had a document tube sitting in his locker overnight. Nobody's interrogating him, because Evan says he doesn't care and everyone believes him. Leo would say that's proof the theatre's a distraction. Leo would say anything that ends the conversation.</t>
+  </si>
+  <si>
+    <t>C12</t>
+  </si>
+  <si>
+    <t>No, and I'll tell you the thing that makes me look bad: after Mira left I moved several tubes around in the loft to keep rain off the paper stock and never updated the inventory. That's sloppy, not sinister. Hana's told me for a year that bad storage and bad access are the same institutional problem. She's right, and I should have listened sooner.</t>
+  </si>
+  <si>
+    <t>W05</t>
+  </si>
+  <si>
+    <t>R12</t>
+  </si>
+  <si>
+    <t>S4</t>
+  </si>
+  <si>
+    <t>Accessibility office until 8:15, then the forum. On the way I passed Martin Ellison in the administrative corridor signing insurance forms for tonight, and Elise Grant leaving with a portfolio; I could see the printed programs stacked inside. That corridor doesn't connect to the archive stacks. Leo and I disagree about most of the plan, and he's right that not every administrator with a folder is up to something.</t>
+  </si>
+  <si>
+    <t>R24</t>
+  </si>
+  <si>
+    <t>I think I do, though Mira understands it better. I've heard the rumour that someone meant to settle it last night with a chemistry test on the ink. That couldn't happen: dating ink needs a sample scraped from the document and about a week of lab work, and I checked for the audit that every chemistry-building door locks at six on event nights. I can't judge the comma myself. Priya would want the timestamps first, and I think that's the sensible order.</t>
+  </si>
+  <si>
+    <t>Students at the forum, and one administrator: Celia Park kept asking how the university would describe the result, and pressing for 'a clean answer' for the Board. Around the same time the event materials stopped saying 'the original Charter' and just said 'the Charter'. That may be ordinary legal caution, as Leo says; he's probably right that it isn't proof of anything by itself.</t>
+  </si>
+  <si>
+    <t>It could be; the loft is dry, which is more than most of the building. I was there for the accessibility audit and noticed tubes had been moved and the inventory sheet didn't match. Jonah would say the loft isn't a public room, and he's right; I'd only add that good storage and good access turn out to be the same problem, which is something he and I agree on.</t>
+  </si>
+  <si>
+    <t>Hana closes her folder. “It is only 'political' to people who won't be locked out of the building. Come back when you want to talk about the building.” She leaves.</t>
+  </si>
+  <si>
+    <t>R09</t>
+  </si>
+  <si>
+    <t>It does, though maybe less than the café does to Evan, and that's fine. Since you'll hear about it: the tube in Evan's locker held catering menus and inventory sheets, and it was there before the forum ended. He and I want different things from this building and we both want people treated decently in it.</t>
+  </si>
+  <si>
+    <t>On the side of a building that lets everyone in. Mira and Jonah are on different sides of the theatre question and I've watched them argue about it, but they agree the Charter must not be damaged or lost. I think that's worth more than either of them realizes, and it's probably why they trust each other.</t>
+  </si>
+  <si>
+    <t>No. I've checked the other obvious suspicion for you, since it's the one Sofia keeps raising: steering-group members don't hold archive credentials at all. They reach the archive through the archivist's office, and nobody used that route last night. Sofia may still be right about their motives; she's just wrong about their access.</t>
+  </si>
+  <si>
+    <t>W07</t>
+  </si>
+  <si>
+    <t>R21</t>
+  </si>
+  <si>
+    <t>Newsroom until ten to nine, comparing old scans, then out for air, then back. At 9:20 a courier dropped off a stiff, document-sized envelope and I signed for it. Who sent it is my business. Leo will tell you that's nothing. Leo would tell you a fire alarm was nothing if it interrupted a pitch.</t>
+  </si>
+  <si>
+    <t>I understand it, and I'd rather be corrected than assumed to. What I can say is this: in the photograph we printed, the disputed mark has sharper edges and a different paper shadow than the surrounding ink. Mira noticed it before I did. I may be wrong about what it means; she and I disagree about whether the examination should go ahead at all, and she's right that a careful result would help everyone.</t>
+  </si>
+  <si>
+    <t>Sofia's tone drops. “I don't name sources. Not for the president, not for you.” She picks up her bag and goes.</t>
+  </si>
+  <si>
+    <t>Jonah told me a poster tube in the loft had got heavier since last night. I asked him not to move it again. He treats the loft like a chapel, which is charming and useless. If he'd run an inventory like a normal person we wouldn't be guessing.</t>
+  </si>
+  <si>
+    <t>It's not a football, it's a record. A source who can read the system tells me the log was edited at 9:17 p.m., after the archive closed. That's not politics, that's a timestamp. Hana keeps saying we should wait for the experts. The experts are examining a document nobody can vouch for.</t>
+  </si>
+  <si>
+    <t>R14</t>
+  </si>
+  <si>
+    <t>It's the only story that matters this year. And yes, I once printed a committee meeting date I hadn't verified. I corrected it the same week, and the newsroom badge log shows I never left the building before 8:50. Nia thinks admitting errors makes people trust you. In my experience it gives administrators a stick.</t>
+  </si>
+  <si>
+    <t>R10</t>
+  </si>
+  <si>
+    <t>The public's. Which is why I'll tell you Martin Ellison, the archivist, was hanging around the archive office at half past eight. Nobody in the administration will explain what he was doing. Evan says he saw nothing unusual. Evan wouldn't notice a fire unless it was in the espresso machine.</t>
+  </si>
+  <si>
+    <t>No. I have something better: there's a small crease near the mark in the older photographs of the Charter. It isn't in the photo we printed of the examination copy. Mira flagged it. Priya says an image needs the same care as a log. Fine. The image says what it says.</t>
+  </si>
+  <si>
+    <t>W08</t>
+  </si>
+  <si>
+    <t>Catered the forum, then the café till close. About five to nine someone carried a long cardboard tube from the Commons toward the theatre; it had theatre paint on one end and nearly took out my sign. Couldn't see the face. Leo says I should have looked harder. Leo has never worked a counter.</t>
+  </si>
+  <si>
+    <t>R16</t>
+  </si>
+  <si>
+    <t>I don't and I don't need to. I delivered coffee to the meeting room where they were arguing about it at 7:20, and Hana was signing in to get a folder while the forum was still going. Mira can explain the comma to you for an hour. It won't make the café stay open.</t>
+  </si>
+  <si>
+    <t>C16</t>
+  </si>
+  <si>
+    <t>Mira, at the counter, around ten to nine. She said she'd 'keep it safe until someone can compare the two'. I didn't ask what 'it' was. Maybe I should have; Sofia would have. She and I want different things from all this, but she's right that people say important things to whoever's pouring the tea.</t>
+  </si>
+  <si>
+    <t>R17</t>
+  </si>
+  <si>
+    <t>Could be. When I locked up I saw a rolled parchment that looked just like the Charter lying on the costume trunk by the stage door. Didn't touch it. Jonah thinks the loft is the last honest room on campus. It's a loft with a leak on the north side.</t>
+  </si>
+  <si>
+    <t>Sure, and it was a football on the table at 7:45 when I was clearing the forum plates: blue folder, seal intact, Nia handed it back to the archive. Then everyone went home to be outraged. Hana would say that's the wrong lesson. Hana would say that about most of my lessons.</t>
+  </si>
+  <si>
+    <t>Evan stops wiping the counter. “You want my observations, then tell me they don't count. Pick one.” He goes into the back.</t>
   </si>
   <si>
     <t>C13</t>
   </si>
   <si>
-    <t>MC3</t>
-  </si>
-  <si>
-    <t>Probably. Around five to nine I saw someone hauling a long cardboard tube from the Commons toward the theatre; it had paint on one end, the way all Jonah's tubes do. Theatre people carry tubes constantly, which is exactly why nobody looks. Jonah will tell you the loft is sacred. It's a fire hazard with a curtain.</t>
-  </si>
-  <si>
-    <t>C09</t>
-  </si>
-  <si>
-    <t>It's been a football since the forum. The event materials changed late; first it was an examination of 'the original Charter', then just 'the Charter', because Celia Park wanted a clean answer for the Board. That's communications people being communications people. Hana reads it as a plot. Hana reads everything as a plot.</t>
-  </si>
-  <si>
-    <t>R01</t>
-  </si>
-  <si>
-    <t>S1</t>
-  </si>
-  <si>
-    <t>Yes, and I'll save you the discovery: the committee told me the club would get first choice of new office space. That makes my support look bought. It isn't. I wanted the building before anyone offered me anything, and no amount of Nia's compromise talk changes the fact that the current Commons is a museum with bad Wi-Fi.</t>
-  </si>
-  <si>
-    <t>R20</t>
-  </si>
-  <si>
-    <t>S8</t>
-  </si>
-  <si>
-    <t>On the side of getting things built. If you want to know whose side people are on, ask who's feeding Sofia's paper: a draft student-government resolution that only a handful of people had was in this morning's edition. Somebody is passing her documents. I'm not going to pretend, like Nia does, that everyone in this is acting in good faith.</t>
-  </si>
-  <si>
-    <t>C01</t>
-  </si>
-  <si>
-    <t>No. I last saw the Charter at the forum at 7:45, in a blue archival folder, seal intact, before it went back to the cabinet. I didn't touch it. Anyone who thinks I'd risk the Board's whole process to steal a document I want examined hasn't thought about it for five seconds. Sofia hasn't.</t>
-  </si>
-  <si>
-    <t>W03</t>
-  </si>
-  <si>
-    <t>C03</t>
-  </si>
-  <si>
-    <t>I was in the lab until about 8:55 with the access dashboard open. The thing worth your time is this: the archive log was edited at 9:17 p.m., after the archive closed at nine, and edits need an archive credential, not maintenance or admin. Leo thinks logs are trivia. That's because he's never read one.</t>
-  </si>
-  <si>
-    <t>Priya's face goes flat. “I wrote the explainer. If you need the comma explained to me, we're finished.” She turns back to her screen.</t>
-  </si>
-  <si>
-    <t>C08</t>
-  </si>
-  <si>
-    <t>Mira, a few days ago. She asked me to compare the newspaper photograph with older images of the Charter. I might be wrong about what it means, but a small crease near the mark that shows in the older photographs isn't in the newspaper one. Mira and I don't agree about facial recognition, and I still think she's right that images deserve the same scrutiny as logs.</t>
-  </si>
-  <si>
-    <t>R18</t>
-  </si>
-  <si>
-    <t>Check the equipment-booking system before you check the gossip. It shows the theatre signed out an item called 'Commons Charter' last week, and it hasn't come back. That's a record, not a rumour. Jonah acts like the loft is off-limits to questions. It's a room.</t>
-  </si>
-  <si>
-    <t>R03</t>
-  </si>
-  <si>
-    <t>It's an evidence question, not a political one. While people are pointing at Leo, the incubator badge reader has him in the business building from 8:36 until after 9:10. He couldn't have been in the archive at 8:42 or at a terminal at 9:17. Sofia would rather run the rumour than the log. That's the difference between us.</t>
-  </si>
-  <si>
-    <t>It matters, though maybe not in the way you'd expect. I care that the system is read correctly: no credential other than Mira's opened the archive between the forum and closing. That doesn't tell you what she did inside, and I'd want to hear her account before drawing a line from a swipe to a theft. Hana's right that a log records entry, not intent.</t>
-  </si>
-  <si>
-    <t>On the side of what the record shows. Mira's credential opened the archive at 8:42; an ordinary entry, no forced door. I know Leo reads that as case closed, and he may turn out to be right. I'd just rather we got there by asking what an ordinary entry means when the person has every right to be there.</t>
-  </si>
-  <si>
-    <t>R04</t>
-  </si>
-  <si>
-    <t>No. I copied a debugging file from the access system without permission, and I regret it, and it's going to come out anyway. It has credential events in it, nothing else. Leo will call it a distraction. Leo calls anything he doesn't understand a distraction.</t>
-  </si>
-  <si>
-    <t>W04</t>
-  </si>
-  <si>
-    <t>R23</t>
-  </si>
-  <si>
-    <t>S9</t>
-  </si>
-  <si>
-    <t>Loading dock from half past seven to nearly nine, wrangling a lighting case. Around twenty to nine Evan slipped out of the café for ten minutes and came back from the direction of the chemistry building, and somebody at the forum had joked that the comma's ink could be tested in a lab tonight. I didn't ask him about it. Leo would say I should have. He might be right; theatre people are so used to things moving that we stop asking.</t>
-  </si>
-  <si>
-    <t>C17</t>
-  </si>
-  <si>
-    <t>I understand it well enough to know why Mira cares. We argue about whether the theatre should block the whole plan, and we probably always will, but on one thing we're the same: the Charter should not get damaged or lost. I might be naïve about the politics. I'm not naïve about paper in a damp building.</t>
-  </si>
-  <si>
-    <t>C12</t>
-  </si>
-  <si>
-    <t>Mira, last night. She needed a container and I gave her an empty poster tube, the one labelled 'Spring Gala 2023'. That's it. Now Sofia is sniffing around the loft as if a cardboard tube proves a conspiracy. She wants a scandal more than she wants an answer.</t>
-  </si>
-  <si>
-    <t>Jonah sets down the cable coil. “So the theatre is your suspect. If you have evidence, show it. If not, stay out of my loft.” He walks away.</t>
-  </si>
-  <si>
-    <t>R15</t>
-  </si>
-  <si>
-    <t>S6</t>
-  </si>
-  <si>
-    <t>Everything is a football to the people kicking it. Want something concrete? Hana went into the steering group's restricted meeting room. I saw her come out with a folder. She'll tell you it was for accessibility. Maybe. She also never misses a chance to make the administration look bad.</t>
-  </si>
-  <si>
-    <t>C14</t>
-  </si>
-  <si>
-    <t>It matters. That 'Spring Gala 2023' tube is up in the scenery loft now, and it's heavier than an empty tube has any business being. I haven't opened it. I should probably admit that Priya's point about chains of custody applies to my loft as much as to her logs, and that I'd feel better if someone from the archive looked before anyone else does.</t>
-  </si>
-  <si>
-    <t>R07</t>
-  </si>
-  <si>
-    <t>S3</t>
-  </si>
-  <si>
-    <t>The theatre's. Since you're asking whose side, ask the café. Evan had a document tube sitting in his locker overnight. Nobody's interrogating him, because Evan says he doesn't care and everyone believes him. Leo would say that's proof the theatre's a distraction. Leo would say anything that ends the conversation.</t>
-  </si>
-  <si>
-    <t>C15</t>
-  </si>
-  <si>
-    <t>No, and I'll tell you the thing that makes me look bad: after Mira left I moved several tubes around in the loft to keep rain off the paper stock and never updated the inventory. That's sloppy, not sinister. Hana's told me for a year that bad storage and bad access are the same institutional problem. She's right, and I should have listened sooner.</t>
-  </si>
-  <si>
-    <t>W05</t>
-  </si>
-  <si>
-    <t>R12</t>
-  </si>
-  <si>
-    <t>S4</t>
-  </si>
-  <si>
-    <t>Accessibility office until 8:15, then the forum. On the way I passed Martin Ellison in the administrative corridor signing insurance forms for tonight, and Elise Grant leaving with a portfolio; I could see the printed programs stacked inside. That corridor doesn't connect to the archive stacks. Leo and I disagree about most of the plan, and he's right that not every administrator with a folder is up to something.</t>
-  </si>
-  <si>
-    <t>R24</t>
-  </si>
-  <si>
-    <t>I think I do, though Mira understands it better. I've heard the rumour that someone meant to settle it last night with a chemistry test on the ink. That couldn't happen: dating ink needs a sample scraped from the document and about a week of lab work, and I checked for the audit that every chemistry-building door locks at six on event nights. I can't judge the comma myself. Priya would want the timestamps first, and I think that's the sensible order.</t>
-  </si>
-  <si>
-    <t>Students at the forum, and one administrator: Celia Park kept asking how the university would describe the result, and pressing for 'a clean answer' for the Board. Around the same time the event materials stopped saying 'the original Charter' and just said 'the Charter'. That may be ordinary legal caution, as Leo says; he's probably right that it isn't proof of anything by itself.</t>
-  </si>
-  <si>
-    <t>It could be; the loft is dry, which is more than most of the building. I was there for the accessibility audit and noticed tubes had been moved and the inventory sheet didn't match. Jonah would say the loft isn't a public room, and he's right; I'd only add that good storage and good access turn out to be the same problem, which is something he and I agree on.</t>
-  </si>
-  <si>
-    <t>Hana closes her folder. “It is only 'political' to people who won't be locked out of the building. Come back when you want to talk about the building.” She leaves.</t>
-  </si>
-  <si>
-    <t>R09</t>
-  </si>
-  <si>
-    <t>It does, though maybe less than the café does to Evan, and that's fine. Since you'll hear about it: the tube in Evan's locker held catering menus and inventory sheets, and it was there before the forum ended. He and I want different things from this building and we both want people treated decently in it.</t>
-  </si>
-  <si>
-    <t>On the side of a building that lets everyone in. Mira and Jonah are on different sides of the theatre question and I've watched them argue about it, but they agree the Charter must not be damaged or lost. I think that's worth more than either of them realizes, and it's probably why they trust each other.</t>
-  </si>
-  <si>
-    <t>No. I've checked the other obvious suspicion for you, since it's the one Sofia keeps raising: steering-group members don't hold archive credentials at all. They reach the archive through the archivist's office, and nobody used that route last night. Sofia may still be right about their motives; she's just wrong about their access.</t>
-  </si>
-  <si>
-    <t>W07</t>
-  </si>
-  <si>
-    <t>R21</t>
-  </si>
-  <si>
-    <t>Newsroom until ten to nine, comparing old scans, then out for air, then back. At 9:20 a courier dropped off a stiff, document-sized envelope and I signed for it. Who sent it is my business. Leo will tell you that's nothing. Leo would tell you a fire alarm was nothing if it interrupted a pitch.</t>
-  </si>
-  <si>
-    <t>I understand it, and I'd rather be corrected than assumed to. What I can say is this: in the photograph we printed, the disputed mark has sharper edges and a different paper shadow than the surrounding ink. Mira noticed it before I did. I may be wrong about what it means; she and I disagree about whether the examination should go ahead at all, and she's right that a careful result would help everyone.</t>
-  </si>
-  <si>
-    <t>Sofia's tone drops. “I don't name sources. Not for the president, not for you.” She picks up her bag and goes.</t>
-  </si>
-  <si>
-    <t>Jonah told me a poster tube in the loft had got heavier since last night. I asked him not to move it again. He treats the loft like a chapel, which is charming and useless. If he'd run an inventory like a normal person we wouldn't be guessing.</t>
-  </si>
-  <si>
-    <t>It's not a football, it's a record. A source who can read the system tells me the log was edited at 9:17 p.m., after the archive closed. That's not politics, that's a timestamp. Hana keeps saying we should wait for the experts. The experts are examining a document nobody can vouch for.</t>
-  </si>
-  <si>
-    <t>R14</t>
-  </si>
-  <si>
-    <t>It's the only story that matters this year. And yes, I once printed a committee meeting date I hadn't verified. I corrected it the same week, and the newsroom badge log shows I never left the building before 8:50. Nia thinks admitting errors makes people trust you. In my experience it gives administrators a stick.</t>
-  </si>
-  <si>
-    <t>R10</t>
-  </si>
-  <si>
-    <t>The public's. Which is why I'll tell you Martin Ellison, the archivist, was hanging around the archive office at half past eight. Nobody in the administration will explain what he was doing. Evan says he saw nothing unusual. Evan wouldn't notice a fire unless it was in the espresso machine.</t>
-  </si>
-  <si>
-    <t>No. I have something better: there's a small crease near the mark in the older photographs of the Charter. It isn't in the photo we printed of the examination copy. Mira flagged it. Priya says an image needs the same care as a log. Fine. The image says what it says.</t>
-  </si>
-  <si>
-    <t>W08</t>
-  </si>
-  <si>
-    <t>Catered the forum, then the café till close. About five to nine someone carried a long cardboard tube from the Commons toward the theatre; it had theatre paint on one end and nearly took out my sign. Couldn't see the face. Leo says I should have looked harder. Leo has never worked a counter.</t>
-  </si>
-  <si>
-    <t>R16</t>
-  </si>
-  <si>
-    <t>I don't and I don't need to. I delivered coffee to the meeting room where they were arguing about it at 7:20, and Hana was signing in to get a folder while the forum was still going. Mira can explain the comma to you for an hour. It won't make the café stay open.</t>
-  </si>
-  <si>
-    <t>C20</t>
-  </si>
-  <si>
-    <t>Mira, at the counter, around ten to nine. She said she'd 'keep it safe until someone can compare the two'. I didn't ask what 'it' was. Maybe I should have; Sofia would have. She and I want different things from all this, but she's right that people say important things to whoever's pouring the tea.</t>
-  </si>
-  <si>
-    <t>R17</t>
-  </si>
-  <si>
-    <t>Could be. When I locked up I saw a rolled parchment that looked just like the Charter lying on the costume trunk by the stage door. Didn't touch it. Jonah thinks the loft is the last honest room on campus. It's a loft with a leak on the north side.</t>
-  </si>
-  <si>
-    <t>Sure, and it was a football on the table at 7:45 when I was clearing the forum plates: blue folder, seal intact, Nia handed it back to the archive. Then everyone went home to be outraged. Hana would say that's the wrong lesson. Hana would say that about most of my lessons.</t>
-  </si>
-  <si>
-    <t>Evan stops wiping the counter. “You want my observations, then tell me they don't count. Pick one.” He goes into the back.</t>
-  </si>
-  <si>
-    <t>C16</t>
-  </si>
-  <si>
     <t>Nobody's. Since you ask fairly: around ten to nine I saw Mira and Jonah talking by the theatre. It looked like two people sorting out where to put something, not an argument. I could be wrong; I was fifty feet away. Nia says everyone in this is on the same side underneath. That's more generous than I'd be, but she might be right.</t>
   </si>
   <si>
@@ -1438,7 +1438,7 @@
     <t>Why it was taken</t>
   </si>
   <si>
-    <t>C06, C07, C08, C09</t>
+    <t>C05, C06, C07, C08</t>
   </si>
   <si>
     <t>Mira has long argued the disputed mark is an original comma. The newspaper photograph of the 'examination copy' shows a mark with the wrong edges and shadow, and a crease seen in older photographs is missing. The event materials quietly stopped calling the object 'the original'. Mira had every reason to believe the document prepared for examination is not the real one.</t>
@@ -1450,7 +1450,7 @@
     <t>Where it is</t>
   </si>
   <si>
-    <t>C12, C13, C14, C15</t>
+    <t>C09, C10, C11, C12</t>
   </si>
   <si>
     <t>Jonah gave Mira an empty poster tube labelled 'Spring Gala 2023'. At about 8:55 a tube with theatre paint on one end was carried from the Commons toward the theatre. That tube is now in the scenery loft, heavier than it should be, and Jonah has since moved tubes around without updating the inventory.</t>
@@ -1462,7 +1462,7 @@
     <t>What it adds up to</t>
   </si>
   <si>
-    <t>C16, C17, C19, C20</t>
+    <t>C13, C14, C15, C16</t>
   </si>
   <si>
     <t>Mira and Jonah met near the theatre for a practical reason: both want the Charter undamaged. The steering group had no archive credential to use that night. Mira means to return the Charter once the examination copy can be compared against it. This was protection, not theft, and it can be resolved before six o'clock.</t>
@@ -1870,7 +1870,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1891,6 +1891,12 @@
     </xf>
     <xf borderId="2" fillId="6" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="2" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3345,7 +3351,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="8" t="s">
         <v>204</v>
       </c>
       <c r="B6" s="2" t="s">
@@ -3359,7 +3365,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="8" t="s">
         <v>226</v>
       </c>
       <c r="B7" s="2" t="s">
@@ -3373,7 +3379,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="8" t="s">
         <v>261</v>
       </c>
       <c r="B8" s="2" t="s">
@@ -3387,7 +3393,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="8" t="s">
         <v>247</v>
       </c>
       <c r="B9" s="2" t="s">
@@ -3401,7 +3407,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="8" t="s">
         <v>277</v>
       </c>
       <c r="B10" s="2" t="s">
@@ -3415,7 +3421,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="8" t="s">
         <v>244</v>
       </c>
       <c r="B11" s="2" t="s">
@@ -3429,7 +3435,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="8" t="s">
         <v>283</v>
       </c>
       <c r="B12" s="2" t="s">
@@ -3443,7 +3449,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="8" t="s">
         <v>288</v>
       </c>
       <c r="B13" s="2" t="s">
@@ -3457,7 +3463,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="8" t="s">
         <v>325</v>
       </c>
       <c r="B14" s="2" t="s">
@@ -3471,7 +3477,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="8" t="s">
         <v>275</v>
       </c>
       <c r="B15" s="2" t="s">
@@ -3485,7 +3491,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="8" t="s">
         <v>221</v>
       </c>
       <c r="B16" s="2" t="s">
@@ -3499,7 +3505,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="8" t="s">
         <v>319</v>
       </c>
       <c r="B17" s="2" t="s">
@@ -4559,7 +4565,7 @@
       <c r="C3" s="2" t="s">
         <v>470</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="8" t="s">
         <v>471</v>
       </c>
       <c r="E3" s="2" t="s">
@@ -4576,7 +4582,7 @@
       <c r="C4" s="2" t="s">
         <v>474</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="8" t="s">
         <v>475</v>
       </c>
       <c r="E4" s="2" t="s">
@@ -4593,7 +4599,7 @@
       <c r="C5" s="2" t="s">
         <v>478</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="8" t="s">
         <v>479</v>
       </c>
       <c r="E5" s="2" t="s">
@@ -12788,7 +12794,7 @@
       <c r="G2" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="7" t="s">
         <v>122</v>
       </c>
       <c r="I2" s="6" t="s">
@@ -12799,7 +12805,7 @@
       <c r="A3" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="7" t="s">
         <v>125</v>
       </c>
       <c r="C3" s="6" t="s">
@@ -12808,19 +12814,19 @@
       <c r="D3" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="7" t="s">
         <v>128</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" s="7" t="s">
         <v>130</v>
       </c>
       <c r="H3" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="I3" s="7" t="s">
         <v>132</v>
       </c>
     </row>
@@ -12834,19 +12840,19 @@
       <c r="C4" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="7" t="s">
         <v>136</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="7" t="s">
         <v>137</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="7" t="s">
         <v>138</v>
       </c>
       <c r="G4" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="H4" s="7" t="s">
         <v>140</v>
       </c>
       <c r="I4" s="4" t="s">
@@ -12860,7 +12866,7 @@
       <c r="B5" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="7" t="s">
         <v>144</v>
       </c>
       <c r="D5" s="4" t="s">
@@ -12869,16 +12875,16 @@
       <c r="E5" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="7" t="s">
         <v>148</v>
       </c>
       <c r="H5" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="I5" s="7" t="s">
         <v>150</v>
       </c>
     </row>
@@ -12886,10 +12892,10 @@
       <c r="A6" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="7" t="s">
         <v>152</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="7" t="s">
         <v>153</v>
       </c>
       <c r="D6" s="6" t="s">
@@ -12915,7 +12921,7 @@
       <c r="A7" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="7" t="s">
         <v>161</v>
       </c>
       <c r="C7" s="6" t="s">
@@ -12924,7 +12930,7 @@
       <c r="D7" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="7" t="s">
         <v>164</v>
       </c>
       <c r="F7" s="6" t="s">
@@ -12936,7 +12942,7 @@
       <c r="H7" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="I7" s="4" t="s">
+      <c r="I7" s="7" t="s">
         <v>168</v>
       </c>
     </row>
@@ -12956,13 +12962,13 @@
       <c r="E8" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="7" t="s">
         <v>174</v>
       </c>
       <c r="G8" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="H8" s="4" t="s">
+      <c r="H8" s="7" t="s">
         <v>176</v>
       </c>
       <c r="I8" s="5" t="s">
@@ -12982,19 +12988,19 @@
       <c r="D9" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="F9" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="G9" s="7" t="s">
         <v>184</v>
       </c>
       <c r="H9" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="I9" s="4" t="s">
+      <c r="I9" s="7" t="s">
         <v>186</v>
       </c>
     </row>
@@ -14076,7 +14082,7 @@
       <c r="D3" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="8" t="s">
         <v>204</v>
       </c>
       <c r="F3" s="2" t="s">
@@ -14163,7 +14169,7 @@
       <c r="D6" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="8" t="s">
         <v>221</v>
       </c>
       <c r="F6" s="2" t="s">
@@ -14192,7 +14198,7 @@
       <c r="D7" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="8" t="s">
         <v>226</v>
       </c>
       <c r="F7" s="2" t="s">
@@ -14358,7 +14364,7 @@
       <c r="D13" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="E13" s="8" t="s">
         <v>244</v>
       </c>
       <c r="F13" s="2" t="s">
@@ -14387,7 +14393,7 @@
       <c r="D14" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="E14" s="8" t="s">
         <v>247</v>
       </c>
       <c r="F14" s="2" t="s">
@@ -14557,7 +14563,7 @@
       <c r="D20" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="E20" s="2" t="s">
+      <c r="E20" s="8" t="s">
         <v>261</v>
       </c>
       <c r="F20" s="2" t="s">
@@ -14760,7 +14766,7 @@
       <c r="D27" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="E27" s="2" t="s">
+      <c r="E27" s="8" t="s">
         <v>275</v>
       </c>
       <c r="F27" s="2" t="s">
@@ -14789,7 +14795,7 @@
       <c r="D28" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="E28" s="2" t="s">
+      <c r="E28" s="8" t="s">
         <v>277</v>
       </c>
       <c r="F28" s="2" t="s">
@@ -14872,7 +14878,7 @@
       <c r="D31" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="E31" s="2" t="s">
+      <c r="E31" s="8" t="s">
         <v>283</v>
       </c>
       <c r="F31" s="2" t="s">
@@ -14930,7 +14936,7 @@
       <c r="D33" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="E33" s="2" t="s">
+      <c r="E33" s="8" t="s">
         <v>288</v>
       </c>
       <c r="F33" s="2" t="s">
@@ -15017,7 +15023,7 @@
       <c r="D36" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="E36" s="2" t="s">
+      <c r="E36" s="8" t="s">
         <v>247</v>
       </c>
       <c r="F36" s="2" t="s">
@@ -15046,7 +15052,7 @@
       <c r="D37" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="E37" s="2" t="s">
+      <c r="E37" s="8" t="s">
         <v>288</v>
       </c>
       <c r="F37" s="2" t="s">
@@ -15129,7 +15135,7 @@
       <c r="D40" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="E40" s="2" t="s">
+      <c r="E40" s="8" t="s">
         <v>275</v>
       </c>
       <c r="F40" s="2" t="s">
@@ -15158,7 +15164,7 @@
       <c r="D41" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="E41" s="2" t="s">
+      <c r="E41" s="8" t="s">
         <v>221</v>
       </c>
       <c r="F41" s="2" t="s">
@@ -15216,7 +15222,7 @@
       <c r="D43" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="E43" s="2" t="s">
+      <c r="E43" s="8" t="s">
         <v>226</v>
       </c>
       <c r="F43" s="2" t="s">
@@ -15270,7 +15276,7 @@
       <c r="D45" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="E45" s="2" t="s">
+      <c r="E45" s="8" t="s">
         <v>283</v>
       </c>
       <c r="F45" s="2" t="s">
@@ -15386,7 +15392,7 @@
       <c r="D49" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="E49" s="2" t="s">
+      <c r="E49" s="8" t="s">
         <v>261</v>
       </c>
       <c r="F49" s="2" t="s">
@@ -15415,7 +15421,7 @@
       <c r="D50" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="E50" s="2" t="s">
+      <c r="E50" s="8" t="s">
         <v>244</v>
       </c>
       <c r="F50" s="2" t="s">
@@ -15473,7 +15479,7 @@
       <c r="D52" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="E52" s="2" t="s">
+      <c r="E52" s="8" t="s">
         <v>319</v>
       </c>
       <c r="F52" s="2" t="s">
@@ -15585,7 +15591,7 @@
       <c r="D56" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="E56" s="2" t="s">
+      <c r="E56" s="8" t="s">
         <v>325</v>
       </c>
       <c r="F56" s="2" t="s">
@@ -15672,7 +15678,7 @@
       <c r="D59" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="E59" s="2" t="s">
+      <c r="E59" s="8" t="s">
         <v>204</v>
       </c>
       <c r="F59" s="2" t="s">
@@ -15730,7 +15736,7 @@
       <c r="D61" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="E61" s="2" t="s">
+      <c r="E61" s="8" t="s">
         <v>277</v>
       </c>
       <c r="F61" s="2" t="s">
@@ -15788,7 +15794,7 @@
       <c r="D63" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="E63" s="2" t="s">
+      <c r="E63" s="8" t="s">
         <v>319</v>
       </c>
       <c r="F63" s="2" t="s">
@@ -15842,7 +15848,7 @@
       <c r="D65" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="E65" s="2" t="s">
+      <c r="E65" s="8" t="s">
         <v>325</v>
       </c>
       <c r="F65" s="2" t="s">

</xml_diff>

<commit_message>
Left-align and italicize the Start pitch; rebuild with updated game text and matrix
Game text Text!C21 (start.intro) and matrix Passages!C2 (pitch) changed in the Google Sheets.
The packet download was left out: it is mid-rewrite and no longer matches the matrix's CCC summary.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scenarios/commons-comma/The Commons' Comma – Response Matrix.xlsx
+++ b/scenarios/commons-comma/The Commons' Comma – Response Matrix.xlsx
@@ -172,7 +172,7 @@
     <t>Summary</t>
   </si>
   <si>
-    <t>The night before the university publicly examines its founding Charter to settle whether a disputed ink mark is a comma, the Charter vanishes from the archive. You have until five o'clock and thirty questions to find out who took it, why, and where it is, by interviewing eight students who each know something and each have an opinion about the renovation the comma would decide.</t>
+    <t>The night before the university publicly examines its founding Charter to settle whether a disputed ink mark is a comma, the Charter vanishes from the archive. You have until five o'clock to find out who took it, why, and where it is, by interviewing eight students who each know something and each have an opinion about the controversial renovation of the commons - which the comma/ink blot would decide.</t>
   </si>
   <si>
     <t>Background/summary shown on the title screen.</t>
@@ -1880,6 +1880,9 @@
     <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
+    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
     <xf borderId="2" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
@@ -1893,9 +1896,6 @@
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="2" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3351,7 +3351,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="3" t="s">
         <v>204</v>
       </c>
       <c r="B6" s="2" t="s">
@@ -3365,7 +3365,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="3" t="s">
         <v>226</v>
       </c>
       <c r="B7" s="2" t="s">
@@ -3379,7 +3379,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="3" t="s">
         <v>261</v>
       </c>
       <c r="B8" s="2" t="s">
@@ -3393,7 +3393,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="3" t="s">
         <v>247</v>
       </c>
       <c r="B9" s="2" t="s">
@@ -3407,7 +3407,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="3" t="s">
         <v>277</v>
       </c>
       <c r="B10" s="2" t="s">
@@ -3421,7 +3421,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="3" t="s">
         <v>244</v>
       </c>
       <c r="B11" s="2" t="s">
@@ -3435,7 +3435,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="s">
+      <c r="A12" s="3" t="s">
         <v>283</v>
       </c>
       <c r="B12" s="2" t="s">
@@ -3449,7 +3449,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="3" t="s">
         <v>288</v>
       </c>
       <c r="B13" s="2" t="s">
@@ -3463,7 +3463,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="s">
+      <c r="A14" s="3" t="s">
         <v>325</v>
       </c>
       <c r="B14" s="2" t="s">
@@ -3477,7 +3477,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="s">
+      <c r="A15" s="3" t="s">
         <v>275</v>
       </c>
       <c r="B15" s="2" t="s">
@@ -3491,7 +3491,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="s">
+      <c r="A16" s="3" t="s">
         <v>221</v>
       </c>
       <c r="B16" s="2" t="s">
@@ -3505,7 +3505,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="s">
+      <c r="A17" s="3" t="s">
         <v>319</v>
       </c>
       <c r="B17" s="2" t="s">
@@ -4565,7 +4565,7 @@
       <c r="C3" s="2" t="s">
         <v>470</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="3" t="s">
         <v>471</v>
       </c>
       <c r="E3" s="2" t="s">
@@ -4582,7 +4582,7 @@
       <c r="C4" s="2" t="s">
         <v>474</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="3" t="s">
         <v>475</v>
       </c>
       <c r="E4" s="2" t="s">
@@ -4599,7 +4599,7 @@
       <c r="C5" s="2" t="s">
         <v>478</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="3" t="s">
         <v>479</v>
       </c>
       <c r="E5" s="2" t="s">
@@ -9375,7 +9375,7 @@
       <c r="B2" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>49</v>
       </c>
       <c r="D2" s="2" t="s">
@@ -12773,234 +12773,234 @@
       </c>
     </row>
     <row r="2" ht="210.0" customHeight="1">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="H2" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="I2" s="7" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="3" ht="210.0" customHeight="1">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="G3" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="I3" s="7" t="s">
+      <c r="I3" s="8" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="4" ht="210.0" customHeight="1">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="H4" s="8" t="s">
         <v>140</v>
       </c>
-      <c r="I4" s="4" t="s">
+      <c r="I4" s="5" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="5" ht="210.0" customHeight="1">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="8" t="s">
         <v>144</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="8" t="s">
         <v>147</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="G5" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="I5" s="7" t="s">
+      <c r="I5" s="8" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="6" ht="210.0" customHeight="1">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="8" t="s">
         <v>152</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="7" t="s">
         <v>154</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="7" t="s">
         <v>155</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="F6" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="I6" s="6" t="s">
+      <c r="I6" s="7" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="7" ht="210.0" customHeight="1">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="8" t="s">
         <v>161</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="8" t="s">
         <v>164</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="G7" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="H7" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="I7" s="7" t="s">
+      <c r="I7" s="8" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="8" ht="210.0" customHeight="1">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="7" t="s">
         <v>170</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="7" t="s">
         <v>173</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="8" t="s">
         <v>174</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="G8" s="7" t="s">
         <v>175</v>
       </c>
-      <c r="H8" s="7" t="s">
+      <c r="H8" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="I8" s="5" t="s">
+      <c r="I8" s="6" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="9" ht="210.0" customHeight="1">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="7" t="s">
         <v>181</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="8" t="s">
         <v>182</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="8" t="s">
         <v>183</v>
       </c>
-      <c r="G9" s="7" t="s">
+      <c r="G9" s="8" t="s">
         <v>184</v>
       </c>
-      <c r="H9" s="6" t="s">
+      <c r="H9" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="I9" s="7" t="s">
+      <c r="I9" s="8" t="s">
         <v>186</v>
       </c>
     </row>
@@ -14082,7 +14082,7 @@
       <c r="D3" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="3" t="s">
         <v>204</v>
       </c>
       <c r="F3" s="2" t="s">
@@ -14169,7 +14169,7 @@
       <c r="D6" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="3" t="s">
         <v>221</v>
       </c>
       <c r="F6" s="2" t="s">
@@ -14198,7 +14198,7 @@
       <c r="D7" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="3" t="s">
         <v>226</v>
       </c>
       <c r="F7" s="2" t="s">
@@ -14364,7 +14364,7 @@
       <c r="D13" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="E13" s="3" t="s">
         <v>244</v>
       </c>
       <c r="F13" s="2" t="s">
@@ -14393,7 +14393,7 @@
       <c r="D14" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="E14" s="3" t="s">
         <v>247</v>
       </c>
       <c r="F14" s="2" t="s">
@@ -14563,7 +14563,7 @@
       <c r="D20" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="E20" s="8" t="s">
+      <c r="E20" s="3" t="s">
         <v>261</v>
       </c>
       <c r="F20" s="2" t="s">
@@ -14766,7 +14766,7 @@
       <c r="D27" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="E27" s="8" t="s">
+      <c r="E27" s="3" t="s">
         <v>275</v>
       </c>
       <c r="F27" s="2" t="s">
@@ -14795,7 +14795,7 @@
       <c r="D28" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="E28" s="8" t="s">
+      <c r="E28" s="3" t="s">
         <v>277</v>
       </c>
       <c r="F28" s="2" t="s">
@@ -14878,7 +14878,7 @@
       <c r="D31" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="E31" s="8" t="s">
+      <c r="E31" s="3" t="s">
         <v>283</v>
       </c>
       <c r="F31" s="2" t="s">
@@ -14936,7 +14936,7 @@
       <c r="D33" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="E33" s="8" t="s">
+      <c r="E33" s="3" t="s">
         <v>288</v>
       </c>
       <c r="F33" s="2" t="s">
@@ -15023,7 +15023,7 @@
       <c r="D36" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="E36" s="8" t="s">
+      <c r="E36" s="3" t="s">
         <v>247</v>
       </c>
       <c r="F36" s="2" t="s">
@@ -15052,7 +15052,7 @@
       <c r="D37" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="E37" s="8" t="s">
+      <c r="E37" s="3" t="s">
         <v>288</v>
       </c>
       <c r="F37" s="2" t="s">
@@ -15135,7 +15135,7 @@
       <c r="D40" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="E40" s="8" t="s">
+      <c r="E40" s="3" t="s">
         <v>275</v>
       </c>
       <c r="F40" s="2" t="s">
@@ -15164,7 +15164,7 @@
       <c r="D41" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="E41" s="8" t="s">
+      <c r="E41" s="3" t="s">
         <v>221</v>
       </c>
       <c r="F41" s="2" t="s">
@@ -15222,7 +15222,7 @@
       <c r="D43" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="E43" s="8" t="s">
+      <c r="E43" s="3" t="s">
         <v>226</v>
       </c>
       <c r="F43" s="2" t="s">
@@ -15276,7 +15276,7 @@
       <c r="D45" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="E45" s="8" t="s">
+      <c r="E45" s="3" t="s">
         <v>283</v>
       </c>
       <c r="F45" s="2" t="s">
@@ -15392,7 +15392,7 @@
       <c r="D49" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="E49" s="8" t="s">
+      <c r="E49" s="3" t="s">
         <v>261</v>
       </c>
       <c r="F49" s="2" t="s">
@@ -15421,7 +15421,7 @@
       <c r="D50" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="E50" s="8" t="s">
+      <c r="E50" s="3" t="s">
         <v>244</v>
       </c>
       <c r="F50" s="2" t="s">
@@ -15479,7 +15479,7 @@
       <c r="D52" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="E52" s="8" t="s">
+      <c r="E52" s="3" t="s">
         <v>319</v>
       </c>
       <c r="F52" s="2" t="s">
@@ -15591,7 +15591,7 @@
       <c r="D56" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="E56" s="8" t="s">
+      <c r="E56" s="3" t="s">
         <v>325</v>
       </c>
       <c r="F56" s="2" t="s">
@@ -15678,7 +15678,7 @@
       <c r="D59" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="E59" s="8" t="s">
+      <c r="E59" s="3" t="s">
         <v>204</v>
       </c>
       <c r="F59" s="2" t="s">
@@ -15736,7 +15736,7 @@
       <c r="D61" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="E61" s="8" t="s">
+      <c r="E61" s="3" t="s">
         <v>277</v>
       </c>
       <c r="F61" s="2" t="s">
@@ -15794,7 +15794,7 @@
       <c r="D63" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="E63" s="8" t="s">
+      <c r="E63" s="3" t="s">
         <v>319</v>
       </c>
       <c r="F63" s="2" t="s">
@@ -15848,7 +15848,7 @@
       <c r="D65" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="E65" s="8" t="s">
+      <c r="E65" s="3" t="s">
         <v>325</v>
       </c>
       <c r="F65" s="2" t="s">

</xml_diff>

<commit_message>
Rebuild from the Google files (2026-10-21)
</commit_message>
<xml_diff>
--- a/scenarios/commons-comma/The Commons' Comma – Response Matrix.xlsx
+++ b/scenarios/commons-comma/The Commons' Comma – Response Matrix.xlsx
@@ -202,7 +202,7 @@
     <t>Situation</t>
   </si>
   <si>
-    <t>You have just started a work-study job as an administrative assistant in the Office of the President. You expected calendars, filing and photocopying. At 9:05 a.m. on your first morning the president closes the office door.</t>
+    <t>You have just started a work-study job as an administrative assistant in the Office of the President, Tricia Tabula. You expected calendars, filing and photocopying. At 9:05 a.m. on your first morning the president closes the office door.</t>
   </si>
   <si>
     <t>Situates the player.</t>
@@ -211,7 +211,7 @@
     <t>Assignment</t>
   </si>
   <si>
-    <t>“At six o'clock tonight, the university will publicly examine the University Charter. I have just learned that the document prepared for examination may not be the original. If that becomes public before we understand it, the university faces a scandal, and the Board may approve a renovation on the strength of falsified evidence. Find out who removed the Charter, why, and where it is now. Talk to the students who were around the Commons last night. Do not alert the press. You have until five.”</t>
+    <t>“As you know, at six o’clock tonight, the university will publicly examine the Charter. Except we can’t. Because the charter is gone - it is missing from the office of the Archivist where it was waiting for today’s examination. This is a complete disaster! At best, this is hugely embarrassing for the university. At worst we have a criminal affair on our hands. I hope this can be resolved quietly and quickly, and I really hope that if the person who removed it is a student - they can put it back quietly before 18:00 tonight so we can avoid the public investigation of a federal crime that will certainly result in expulsion and probably also criminal charges. You have a chance to save a student from their own foolishness! If it is a student… Talk to the students who were around the Commons last night… see if you can find who removed the Charter! If you find them by five, I promise I’ll do my best to keep this story under wraps. If not… well heaven help us all.”</t>
   </si>
   <si>
     <t>The task and the time pressure, from whoever gives the mystery. Also in the Case file.</t>
@@ -9437,7 +9437,7 @@
       <c r="B3" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="4" t="s">
         <v>59</v>
       </c>
       <c r="D3" s="2" t="s">

</xml_diff>

<commit_message>
Read the witnesses' Background column instead of Role
The matrix's Witnesses sheet now calls the column "Background", as the
packet's Table 4.1 does, and takes its wording from that table. Q2, Q5
and Q7 now use the packet's Table 5.2 wording. Rebuilt with fresh
downloads; the copies of the matrix and packet are refreshed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0164uDwp7jKcQiu9biCMvXzF
</commit_message>
<xml_diff>
--- a/scenarios/commons-comma/The Commons' Comma – Response Matrix.xlsx
+++ b/scenarios/commons-comma/The Commons' Comma – Response Matrix.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1309" uniqueCount="604">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1309" uniqueCount="598">
   <si>
     <t>Sheet</t>
   </si>
@@ -446,7 +446,7 @@
     <t>[C13 | unreceptive] I dropped off the student-government petition at the archive at 7:40 and watched Mr. Ellison put the Charter back in the cabinet and lock up at 7:45. Then the café, like everyone else, until late. Leo will tell you a petition is a waste of paper. Leo has never read one.</t>
   </si>
   <si>
-    <t>Q2. So, what's the deal with the comma? How come it makes such a big difference? Explain to me please.</t>
+    <t>Q2. What's the deal with the comma? How come it makes such a big difference? Explain to me please.</t>
   </si>
   <si>
     <t>[C11 | receptive] I'll try, though I may be too close to it. If that mark is a comma, students approve in their own right; if it's a blot, the house masters can approve for us. What worries me more is the object. I've spent two years with pictures of the Charter going back centuries, and every one shows a small crease running near that mark. I could be wrong about what that means. Priya would say check the evidence before the theory, and she's right.</t>
@@ -527,7 +527,7 @@
     <t>[C05 | unreceptive] They'd gain a delay, and they're welcome to it; the real question is why nobody asked students in the first place. As for their organizer: Jonah's spacey, he leaves things everywhere, and the whole campus knows it. Jonah acts as if the theater is the only thing the renovation threatens. It threatens every student who was never asked.</t>
   </si>
   <si>
-    <t>Q5. Lots of students are only here for four years and then gone. Why should a fight over this Charter matter to you personally?</t>
+    <t>Q5. Students are only here for four years and then they are gone. Why does the fight over the Charter matter to you personally?</t>
   </si>
   <si>
     <t>[R04 | unreceptive] Because the Charter is older than any of us and will outlast all of us; that's the point. And it matters to Sofia too, apparently. She was at the next table in the café when I told Hana and Priya about the missing crease, and she hasn't printed a word since. Hana keeps telling everyone to calm down and wait for the experts. Waiting is how this administration wins.</t>
@@ -581,7 +581,7 @@
     <t>[C14 | unreceptive] The administration will get the answer it paid for. I sit on the archive access committee, so I've seen the log: after 7:45 p.m. the only entry is Mira Shah's credential, at 8:42. Mira thinks the experts will save us. Experts appointed by the administration don't save anyone.</t>
   </si>
   <si>
-    <t>Q7. What's your take on the renovation? Is that a good idea?</t>
+    <t>Q7. What's your take on the renovation of the commons? Is that a good idea?</t>
   </si>
   <si>
     <t>[R24 | receptive] I think the plan loses something we can't rebuild, though I can see why Leo wants rooms that work. People keep saying someone could just test the ink in a chemistry lab and settle the comma. It doesn't work that way: dating ink needs a sample scraped off the document and about a week of lab work, and the chemistry building locks at 6 p.m. anyway. I'd want the experts to have the real object, whatever they find.</t>
@@ -683,7 +683,7 @@
     <t>Q2</t>
   </si>
   <si>
-    <t>So, what's the deal with the comma? How come it makes such a big difference? Explain to me please.</t>
+    <t>What's the deal with the comma? How come it makes such a big difference? Explain to me please.</t>
   </si>
   <si>
     <t>C11</t>
@@ -731,7 +731,7 @@
     <t>Q5</t>
   </si>
   <si>
-    <t>Lots of students are only here for four years and then gone. Why should a fight over this Charter matter to you personally?</t>
+    <t>Students are only here for four years and then they are gone. Why does the fight over the Charter matter to you personally?</t>
   </si>
   <si>
     <t>R04</t>
@@ -758,7 +758,7 @@
     <t>Q7</t>
   </si>
   <si>
-    <t>What's your take on the renovation? Is that a good idea?</t>
+    <t>What's your take on the renovation of the commons? Is that a good idea?</t>
   </si>
   <si>
     <t>R24</t>
@@ -1103,7 +1103,7 @@
     <t>Name</t>
   </si>
   <si>
-    <t>Role</t>
+    <t>Background</t>
   </si>
   <si>
     <t>Public background card</t>
@@ -1136,7 +1136,7 @@
     <t>Portrait</t>
   </si>
   <si>
-    <t>History major; research assistant at the archives.</t>
+    <t>History major, RA at the archives</t>
   </si>
   <si>
     <t>Careful, exact, slow to make claims she cannot support. Preservationist: the Commons is a record of student life. Has argued publicly for months that the disputed mark is an original comma. Works evenings in the archive and studies at the Commons café.</t>
@@ -1157,7 +1157,7 @@
     <t>mira-shah.png</t>
   </si>
   <si>
-    <t>Business major; president of the entrepreneurship club.</t>
+    <t>Business major, president of the entrepreneurship club.</t>
   </si>
   <si>
     <t>Brisk, confident, checks his watch. Treats time as the scarcest resource on campus. Strong supporter of the renovation: students need usable places to build things. Was on the invitation list for tonight's event.</t>
@@ -1178,7 +1178,7 @@
     <t>leo-martinez.png</t>
   </si>
   <si>
-    <t>Computer-science major; research assistant on the campus access-control system.</t>
+    <t>Computer-science major, research assistant on the campus access-control system</t>
   </si>
   <si>
     <t>Precise and technical; explains things once and expects to be understood. Supports the technology in the plan but opposes facial recognition. Wrote the student explainer on how the archive's access system works.</t>
@@ -1199,7 +1199,7 @@
     <t>priya-nwosu.png</t>
   </si>
   <si>
-    <t>Theater major; organizer in the Green Commons Coalition.</t>
+    <t>Theater major, organizer in the Green Commons</t>
   </si>
   <si>
     <t>Wry, warm and easily distracted. Organizes for the Green Commons Coalition because the plan takes rehearsal and storage space that already works. Does his work at the Commons café and is making the posters for the spring production of H.M.S. Pinafore.</t>
@@ -1220,7 +1220,7 @@
     <t>jonah-reed.png</t>
   </si>
   <si>
-    <t>International student; runs the campus accessibility audit.</t>
+    <t>International student</t>
   </si>
   <si>
     <t>Measured, organized, always looking for the practical consequence. Wants ramps, lifts and accessible rooms from the renovation, and no surveillance or privatization with them. Spent last night at the Commons café working on the accessibility audit of campus buildings.</t>
@@ -1259,7 +1259,7 @@
     <t>sofia-alvarez.png</t>
   </si>
   <si>
-    <t>Chemistry major; works the night shift at the Commons café.</t>
+    <t>Chemistry major, works the night shift at the Commons café</t>
   </si>
   <si>
     <t>Laconic, observant, uninterested in campus politics. Works the night shift at the Commons café and sees everyone who comes and goes.</t>
@@ -1280,7 +1280,7 @@
     <t>evan-cho.png</t>
   </si>
   <si>
-    <t>Senior; student-government representative.</t>
+    <t>A senior, student-government representative.</t>
   </si>
   <si>
     <t>Earnest and procedural; a senior who has sat through every consultation the administration skipped. Against the renovation on process grounds: the students must be asked. Sits on the archive access committee.</t>
@@ -1301,27 +1301,15 @@
     <t>nia-williams.png</t>
   </si>
   <si>
-    <t>Background</t>
-  </si>
-  <si>
     <t>Position on the CCA</t>
   </si>
   <si>
-    <t>History major, RA at the archives</t>
-  </si>
-  <si>
     <t>Assets/Witness portraits/mira-shah.png</t>
   </si>
   <si>
-    <t>Business major, president of the entrepreneurship club.</t>
-  </si>
-  <si>
     <t>Assets/Witness portraits/leo-martinez.png</t>
   </si>
   <si>
-    <t>Computer-science major, research assistant on the campus access-control system</t>
-  </si>
-  <si>
     <t>Assets/Witness portraits/priya-nwosu.png</t>
   </si>
   <si>
@@ -1334,9 +1322,6 @@
     <t>Assets/Witness portraits/jonah-reed.png</t>
   </si>
   <si>
-    <t>International student</t>
-  </si>
-  <si>
     <t>Assets/Witness portraits/hana-petrov.png</t>
   </si>
   <si>
@@ -1347,9 +1332,6 @@
   </si>
   <si>
     <t>Assets/Witness portraits/evan-cho.png</t>
-  </si>
-  <si>
-    <t>A senior, student-government representative.</t>
   </si>
   <si>
     <t>Q1, Q2, Q3, Q4, Q6, Q8</t>
@@ -1975,6 +1957,9 @@
     <xf borderId="2" fillId="6" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
+    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -1989,9 +1974,6 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3459,14 +3441,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="9" t="s">
         <v>357</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="9" t="s">
         <v>130</v>
       </c>
-      <c r="C1" s="14" t="s">
-        <v>444</v>
+      <c r="C1" s="9" t="s">
+        <v>438</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -4582,13 +4564,13 @@
         <v>357</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>446</v>
+        <v>440</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>447</v>
+        <v>441</v>
       </c>
     </row>
     <row r="2">
@@ -4599,10 +4581,10 @@
         <v>259</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>448</v>
+        <v>442</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>449</v>
+        <v>443</v>
       </c>
     </row>
     <row r="3">
@@ -4613,10 +4595,10 @@
         <v>259</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>450</v>
+        <v>444</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>451</v>
+        <v>445</v>
       </c>
     </row>
     <row r="4">
@@ -4627,10 +4609,10 @@
         <v>259</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>452</v>
+        <v>446</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>453</v>
+        <v>447</v>
       </c>
     </row>
     <row r="5">
@@ -4641,10 +4623,10 @@
         <v>259</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>454</v>
+        <v>448</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>455</v>
+        <v>449</v>
       </c>
     </row>
     <row r="6">
@@ -4655,10 +4637,10 @@
         <v>262</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>456</v>
+        <v>450</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>457</v>
+        <v>451</v>
       </c>
     </row>
     <row r="7">
@@ -4669,10 +4651,10 @@
         <v>262</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>458</v>
+        <v>452</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>459</v>
+        <v>453</v>
       </c>
     </row>
     <row r="8">
@@ -4683,10 +4665,10 @@
         <v>262</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>460</v>
+        <v>454</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>461</v>
+        <v>455</v>
       </c>
     </row>
     <row r="9">
@@ -4697,10 +4679,10 @@
         <v>262</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>462</v>
+        <v>456</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>463</v>
+        <v>457</v>
       </c>
     </row>
     <row r="10">
@@ -4711,10 +4693,10 @@
         <v>221</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>464</v>
+        <v>458</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>465</v>
+        <v>459</v>
       </c>
     </row>
     <row r="11">
@@ -4725,10 +4707,10 @@
         <v>221</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>466</v>
+        <v>460</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>467</v>
+        <v>461</v>
       </c>
     </row>
     <row r="12">
@@ -4739,10 +4721,10 @@
         <v>221</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>468</v>
+        <v>462</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>469</v>
+        <v>463</v>
       </c>
     </row>
     <row r="13">
@@ -4753,10 +4735,10 @@
         <v>221</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>470</v>
+        <v>464</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>471</v>
+        <v>465</v>
       </c>
     </row>
     <row r="14">
@@ -4767,10 +4749,10 @@
         <v>216</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>472</v>
+        <v>466</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>473</v>
+        <v>467</v>
       </c>
     </row>
     <row r="15">
@@ -4781,10 +4763,10 @@
         <v>216</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>474</v>
+        <v>468</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>475</v>
+        <v>469</v>
       </c>
     </row>
     <row r="16">
@@ -4795,10 +4777,10 @@
         <v>216</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>476</v>
+        <v>470</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>477</v>
+        <v>471</v>
       </c>
     </row>
     <row r="17">
@@ -4809,10 +4791,10 @@
         <v>216</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>478</v>
+        <v>472</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>479</v>
+        <v>473</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -5823,7 +5805,7 @@
         <v>357</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>480</v>
+        <v>474</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>30</v>
@@ -5832,7 +5814,7 @@
         <v>19</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>481</v>
+        <v>475</v>
       </c>
     </row>
     <row r="2">
@@ -5840,16 +5822,16 @@
         <v>259</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>482</v>
+        <v>476</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>483</v>
+        <v>477</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>484</v>
+        <v>478</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>485</v>
+        <v>479</v>
       </c>
     </row>
     <row r="3">
@@ -5857,16 +5839,16 @@
         <v>262</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>486</v>
+        <v>480</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>487</v>
+        <v>481</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>489</v>
+        <v>483</v>
       </c>
     </row>
     <row r="4">
@@ -5874,16 +5856,16 @@
         <v>221</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>490</v>
+        <v>484</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>491</v>
+        <v>485</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>492</v>
+        <v>486</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>493</v>
+        <v>487</v>
       </c>
     </row>
     <row r="5">
@@ -5891,16 +5873,16 @@
         <v>216</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>494</v>
+        <v>488</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>495</v>
+        <v>489</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>496</v>
+        <v>490</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>497</v>
+        <v>491</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -6911,19 +6893,19 @@
         <v>357</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>498</v>
+        <v>492</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>499</v>
+        <v>493</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>500</v>
+        <v>494</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>447</v>
+        <v>441</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>501</v>
+        <v>495</v>
       </c>
     </row>
     <row r="2">
@@ -6934,16 +6916,16 @@
         <v>267</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>502</v>
+        <v>496</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>503</v>
+        <v>497</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>504</v>
+        <v>498</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
     </row>
     <row r="3">
@@ -6954,16 +6936,16 @@
         <v>267</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>502</v>
+        <v>496</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>506</v>
+        <v>500</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>507</v>
+        <v>501</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
     </row>
     <row r="4">
@@ -6974,16 +6956,16 @@
         <v>267</v>
       </c>
       <c r="C4" s="4" t="s">
+        <v>496</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>508</v>
-      </c>
       <c r="E4" s="4" t="s">
-        <v>509</v>
+        <v>503</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
     </row>
     <row r="5">
@@ -6994,16 +6976,16 @@
         <v>237</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>510</v>
+        <v>504</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>511</v>
+        <v>505</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>512</v>
+        <v>506</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>513</v>
+        <v>507</v>
       </c>
     </row>
     <row r="6">
@@ -7014,16 +6996,16 @@
         <v>237</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>510</v>
+        <v>504</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>514</v>
+        <v>508</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>515</v>
+        <v>509</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>513</v>
+        <v>507</v>
       </c>
     </row>
     <row r="7">
@@ -7034,16 +7016,16 @@
         <v>237</v>
       </c>
       <c r="C7" s="4" t="s">
+        <v>504</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>510</v>
       </c>
-      <c r="D7" s="4" t="s">
-        <v>516</v>
-      </c>
       <c r="E7" s="4" t="s">
-        <v>517</v>
+        <v>511</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>513</v>
+        <v>507</v>
       </c>
     </row>
     <row r="8">
@@ -7054,16 +7036,16 @@
         <v>311</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>518</v>
+        <v>512</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>519</v>
+        <v>513</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>520</v>
+        <v>514</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>521</v>
+        <v>515</v>
       </c>
     </row>
     <row r="9">
@@ -7074,16 +7056,16 @@
         <v>311</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>518</v>
+        <v>512</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>522</v>
+        <v>516</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>523</v>
+        <v>517</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>521</v>
+        <v>515</v>
       </c>
     </row>
     <row r="10">
@@ -7094,16 +7076,16 @@
         <v>311</v>
       </c>
       <c r="C10" s="4" t="s">
+        <v>512</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>518</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>524</v>
-      </c>
       <c r="E10" s="4" t="s">
-        <v>525</v>
+        <v>519</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>521</v>
+        <v>515</v>
       </c>
     </row>
     <row r="11">
@@ -7114,16 +7096,16 @@
         <v>285</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>526</v>
+        <v>520</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>527</v>
+        <v>521</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>528</v>
+        <v>522</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>529</v>
+        <v>523</v>
       </c>
     </row>
     <row r="12">
@@ -7134,16 +7116,16 @@
         <v>285</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>526</v>
+        <v>520</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>530</v>
+        <v>524</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>531</v>
+        <v>525</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>529</v>
+        <v>523</v>
       </c>
     </row>
     <row r="13">
@@ -7154,16 +7136,16 @@
         <v>285</v>
       </c>
       <c r="C13" s="4" t="s">
+        <v>520</v>
+      </c>
+      <c r="D13" s="4" t="s">
         <v>526</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>532</v>
-      </c>
       <c r="E13" s="4" t="s">
-        <v>533</v>
+        <v>527</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>529</v>
+        <v>523</v>
       </c>
     </row>
     <row r="14">
@@ -7174,16 +7156,16 @@
         <v>303</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>534</v>
+        <v>528</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>535</v>
+        <v>529</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>536</v>
+        <v>530</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>537</v>
+        <v>531</v>
       </c>
     </row>
     <row r="15">
@@ -7194,16 +7176,16 @@
         <v>303</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>534</v>
+        <v>528</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>538</v>
+        <v>532</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>539</v>
+        <v>533</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>537</v>
+        <v>531</v>
       </c>
     </row>
     <row r="16">
@@ -7214,16 +7196,16 @@
         <v>295</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>540</v>
+        <v>534</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>541</v>
+        <v>535</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>542</v>
+        <v>536</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>543</v>
+        <v>537</v>
       </c>
     </row>
     <row r="17">
@@ -7234,16 +7216,16 @@
         <v>295</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>540</v>
+        <v>534</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>544</v>
+        <v>538</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>545</v>
+        <v>539</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>543</v>
+        <v>537</v>
       </c>
     </row>
     <row r="18">
@@ -7254,16 +7236,16 @@
         <v>232</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>546</v>
+        <v>540</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>547</v>
+        <v>541</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>548</v>
+        <v>542</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>549</v>
+        <v>543</v>
       </c>
     </row>
     <row r="19">
@@ -7274,16 +7256,16 @@
         <v>232</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>546</v>
+        <v>540</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>550</v>
+        <v>544</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>551</v>
+        <v>545</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>549</v>
+        <v>543</v>
       </c>
     </row>
     <row r="20">
@@ -7294,16 +7276,16 @@
         <v>232</v>
       </c>
       <c r="C20" s="4" t="s">
+        <v>540</v>
+      </c>
+      <c r="D20" s="4" t="s">
         <v>546</v>
       </c>
-      <c r="D20" s="4" t="s">
-        <v>552</v>
-      </c>
       <c r="E20" s="4" t="s">
-        <v>553</v>
+        <v>547</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>549</v>
+        <v>543</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
@@ -7314,16 +7296,16 @@
         <v>256</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>554</v>
+        <v>548</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>555</v>
+        <v>549</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>556</v>
+        <v>550</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>557</v>
+        <v>551</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
@@ -7334,16 +7316,16 @@
         <v>256</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>554</v>
+        <v>548</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>558</v>
+        <v>552</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>559</v>
+        <v>553</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>557</v>
+        <v>551</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
@@ -7354,16 +7336,16 @@
         <v>256</v>
       </c>
       <c r="C23" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="D23" s="4" t="s">
         <v>554</v>
       </c>
-      <c r="D23" s="4" t="s">
-        <v>560</v>
-      </c>
       <c r="E23" s="4" t="s">
-        <v>561</v>
+        <v>555</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>557</v>
+        <v>551</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
@@ -7374,16 +7356,16 @@
         <v>246</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>562</v>
+        <v>556</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>563</v>
+        <v>557</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>564</v>
+        <v>558</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>565</v>
+        <v>559</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
@@ -7394,16 +7376,16 @@
         <v>246</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>562</v>
+        <v>556</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>566</v>
+        <v>560</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>567</v>
+        <v>561</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>565</v>
+        <v>559</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1"/>
@@ -8412,16 +8394,16 @@
         <v>204</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>568</v>
+        <v>562</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>569</v>
+        <v>563</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>570</v>
+        <v>564</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>571</v>
+        <v>565</v>
       </c>
     </row>
     <row r="2">
@@ -8432,16 +8414,16 @@
         <v>105</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>572</v>
+        <v>566</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>573</v>
+        <v>567</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>574</v>
+        <v>568</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>575</v>
+        <v>569</v>
       </c>
     </row>
     <row r="3">
@@ -8452,16 +8434,16 @@
         <v>106</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>576</v>
+        <v>570</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>577</v>
+        <v>571</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>578</v>
+        <v>572</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>579</v>
+        <v>573</v>
       </c>
     </row>
     <row r="4">
@@ -8472,16 +8454,16 @@
         <v>107</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>580</v>
+        <v>574</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>581</v>
+        <v>575</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>582</v>
+        <v>576</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>583</v>
+        <v>577</v>
       </c>
     </row>
     <row r="5">
@@ -8492,16 +8474,16 @@
         <v>108</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>584</v>
+        <v>578</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>585</v>
+        <v>579</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>586</v>
+        <v>580</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>587</v>
+        <v>581</v>
       </c>
     </row>
     <row r="6">
@@ -8512,16 +8494,16 @@
         <v>109</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>588</v>
+        <v>582</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>589</v>
+        <v>583</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>590</v>
+        <v>584</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>591</v>
+        <v>585</v>
       </c>
     </row>
     <row r="7">
@@ -8532,16 +8514,16 @@
         <v>110</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>592</v>
+        <v>586</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>593</v>
+        <v>587</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>594</v>
+        <v>588</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>595</v>
+        <v>589</v>
       </c>
     </row>
     <row r="8">
@@ -8552,16 +8534,16 @@
         <v>111</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>596</v>
+        <v>590</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>597</v>
+        <v>591</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>598</v>
+        <v>592</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>599</v>
+        <v>593</v>
       </c>
     </row>
     <row r="9">
@@ -8572,16 +8554,16 @@
         <v>113</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>600</v>
+        <v>594</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>601</v>
+        <v>595</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>602</v>
+        <v>596</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>603</v>
+        <v>597</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -18204,7 +18186,7 @@
       <c r="B1" s="1" t="s">
         <v>358</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="9" t="s">
         <v>359</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -19571,237 +19553,237 @@
   </cols>
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="10" t="s">
         <v>357</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="10" t="s">
         <v>358</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="10" t="s">
+        <v>359</v>
+      </c>
+      <c r="D1" s="10" t="s">
         <v>425</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="E1" s="10" t="s">
+        <v>368</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>366</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>367</v>
+      </c>
+      <c r="H1" s="10" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="2" ht="22.5" customHeight="1">
+      <c r="A2" s="11" t="s">
+        <v>211</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>370</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>372</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>375</v>
+      </c>
+      <c r="F2" s="12">
+        <v>3.0</v>
+      </c>
+      <c r="G2" s="13" t="s">
+        <v>374</v>
+      </c>
+      <c r="H2" s="14" t="s">
         <v>426</v>
       </c>
-      <c r="E1" s="9" t="s">
-        <v>368</v>
-      </c>
-      <c r="F1" s="9" t="s">
-        <v>366</v>
-      </c>
-      <c r="G1" s="9" t="s">
-        <v>367</v>
-      </c>
-      <c r="H1" s="9" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="2" ht="22.5" customHeight="1">
-      <c r="A2" s="10" t="s">
-        <v>211</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="C2" s="10" t="s">
+    </row>
+    <row r="3" ht="22.5" customHeight="1">
+      <c r="A3" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>377</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>379</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>382</v>
+      </c>
+      <c r="F3" s="12">
+        <v>6.0</v>
+      </c>
+      <c r="G3" s="13" t="s">
+        <v>381</v>
+      </c>
+      <c r="H3" s="14" t="s">
         <v>427</v>
       </c>
-      <c r="D2" s="10" t="s">
-        <v>372</v>
-      </c>
-      <c r="E2" s="10" t="s">
-        <v>375</v>
-      </c>
-      <c r="F2" s="11">
-        <v>3.0</v>
-      </c>
-      <c r="G2" s="12" t="s">
-        <v>374</v>
-      </c>
-      <c r="H2" s="13" t="s">
+    </row>
+    <row r="4" ht="22.5" customHeight="1">
+      <c r="A4" s="11" t="s">
+        <v>273</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>384</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>386</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>389</v>
+      </c>
+      <c r="F4" s="12">
+        <v>5.0</v>
+      </c>
+      <c r="G4" s="13" t="s">
+        <v>388</v>
+      </c>
+      <c r="H4" s="14" t="s">
         <v>428</v>
       </c>
     </row>
-    <row r="3" ht="22.5" customHeight="1">
-      <c r="A3" s="10" t="s">
-        <v>253</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>106</v>
-      </c>
-      <c r="C3" s="10" t="s">
+    <row r="5" ht="22.5" customHeight="1">
+      <c r="A5" s="11" t="s">
+        <v>289</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="C5" s="11" t="s">
         <v>429</v>
       </c>
-      <c r="D3" s="10" t="s">
-        <v>379</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>382</v>
-      </c>
-      <c r="F3" s="11">
-        <v>6.0</v>
-      </c>
-      <c r="G3" s="12" t="s">
-        <v>381</v>
-      </c>
-      <c r="H3" s="13" t="s">
+      <c r="D5" s="11" t="s">
+        <v>393</v>
+      </c>
+      <c r="E5" s="11" t="s">
         <v>430</v>
       </c>
-    </row>
-    <row r="4" ht="22.5" customHeight="1">
-      <c r="A4" s="10" t="s">
-        <v>273</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>107</v>
-      </c>
-      <c r="C4" s="10" t="s">
+      <c r="F5" s="12">
+        <v>4.0</v>
+      </c>
+      <c r="G5" s="13" t="s">
+        <v>395</v>
+      </c>
+      <c r="H5" s="14" t="s">
         <v>431</v>
       </c>
-      <c r="D4" s="10" t="s">
-        <v>386</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>389</v>
-      </c>
-      <c r="F4" s="11">
-        <v>5.0</v>
-      </c>
-      <c r="G4" s="12" t="s">
-        <v>388</v>
-      </c>
-      <c r="H4" s="13" t="s">
+    </row>
+    <row r="6" ht="22.5" customHeight="1">
+      <c r="A6" s="11" t="s">
+        <v>306</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>398</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>400</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>403</v>
+      </c>
+      <c r="F6" s="12">
+        <v>1.0</v>
+      </c>
+      <c r="G6" s="13" t="s">
+        <v>402</v>
+      </c>
+      <c r="H6" s="14" t="s">
         <v>432</v>
       </c>
     </row>
-    <row r="5" ht="22.5" customHeight="1">
-      <c r="A5" s="10" t="s">
-        <v>289</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>108</v>
-      </c>
-      <c r="C5" s="10" t="s">
+    <row r="7" ht="22.5" customHeight="1">
+      <c r="A7" s="11" t="s">
+        <v>319</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>405</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>407</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>409</v>
+      </c>
+      <c r="F7" s="12">
+        <v>7.0</v>
+      </c>
+      <c r="G7" s="13" t="s">
+        <v>218</v>
+      </c>
+      <c r="H7" s="14" t="s">
         <v>433</v>
       </c>
-      <c r="D5" s="10" t="s">
-        <v>393</v>
-      </c>
-      <c r="E5" s="10" t="s">
+    </row>
+    <row r="8" ht="22.5" customHeight="1">
+      <c r="A8" s="11" t="s">
+        <v>331</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="C8" s="11" t="s">
         <v>434</v>
       </c>
-      <c r="F5" s="11">
-        <v>4.0</v>
-      </c>
-      <c r="G5" s="12" t="s">
-        <v>395</v>
-      </c>
-      <c r="H5" s="13" t="s">
+      <c r="D8" s="11" t="s">
+        <v>413</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>416</v>
+      </c>
+      <c r="F8" s="12">
+        <v>8.0</v>
+      </c>
+      <c r="G8" s="13" t="s">
+        <v>422</v>
+      </c>
+      <c r="H8" s="14" t="s">
         <v>435</v>
       </c>
     </row>
-    <row r="6" ht="22.5" customHeight="1">
-      <c r="A6" s="10" t="s">
-        <v>306</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>109</v>
-      </c>
-      <c r="C6" s="10" t="s">
+    <row r="9" ht="22.5" customHeight="1">
+      <c r="A9" s="11" t="s">
+        <v>345</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>418</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>420</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>423</v>
+      </c>
+      <c r="F9" s="12">
+        <v>2.0</v>
+      </c>
+      <c r="G9" s="13" t="s">
         <v>436</v>
       </c>
-      <c r="D6" s="10" t="s">
-        <v>400</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>403</v>
-      </c>
-      <c r="F6" s="11">
-        <v>1.0</v>
-      </c>
-      <c r="G6" s="12" t="s">
-        <v>402</v>
-      </c>
-      <c r="H6" s="13" t="s">
+      <c r="H9" s="14" t="s">
         <v>437</v>
-      </c>
-    </row>
-    <row r="7" ht="22.5" customHeight="1">
-      <c r="A7" s="10" t="s">
-        <v>319</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>405</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>407</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>409</v>
-      </c>
-      <c r="F7" s="11">
-        <v>7.0</v>
-      </c>
-      <c r="G7" s="12" t="s">
-        <v>218</v>
-      </c>
-      <c r="H7" s="13" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="8" ht="22.5" customHeight="1">
-      <c r="A8" s="10" t="s">
-        <v>331</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>111</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>439</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>413</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>416</v>
-      </c>
-      <c r="F8" s="11">
-        <v>8.0</v>
-      </c>
-      <c r="G8" s="12" t="s">
-        <v>422</v>
-      </c>
-      <c r="H8" s="13" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="9" ht="22.5" customHeight="1">
-      <c r="A9" s="10" t="s">
-        <v>345</v>
-      </c>
-      <c r="B9" s="10" t="s">
-        <v>113</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>441</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>420</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>423</v>
-      </c>
-      <c r="F9" s="11">
-        <v>2.0</v>
-      </c>
-      <c r="G9" s="12" t="s">
-        <v>442</v>
-      </c>
-      <c r="H9" s="13" t="s">
-        <v>443</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Jonah's location: Theater loft, as the packet's Table 4.3 now says
Matrix Witnesses!L5 updated to match the packet. Rebuilt with fresh
downloads; the packet copy also carries the pending suggestions that
list the withheld secrets under Table 4.3 and delete "The Witnesses in
detail".

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0164uDwp7jKcQiu9biCMvXzF
</commit_message>
<xml_diff>
--- a/scenarios/commons-comma/The Commons' Comma – Response Matrix.xlsx
+++ b/scenarios/commons-comma/The Commons' Comma – Response Matrix.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1309" uniqueCount="598">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1308" uniqueCount="596">
   <si>
     <t>Sheet</t>
   </si>
@@ -1214,7 +1214,7 @@
     <t>Q1, Q2, Q6, Q8</t>
   </si>
   <si>
-    <t>Theater loading dock</t>
+    <t>Theater loft</t>
   </si>
   <si>
     <t>jonah-reed.png</t>
@@ -1301,9 +1301,6 @@
     <t>nia-williams.png</t>
   </si>
   <si>
-    <t>Position on the CCA</t>
-  </si>
-  <si>
     <t>Assets/Witness portraits/mira-shah.png</t>
   </si>
   <si>
@@ -1332,9 +1329,6 @@
   </si>
   <si>
     <t>Assets/Witness portraits/evan-cho.png</t>
-  </si>
-  <si>
-    <t>Q1, Q2, Q3, Q4, Q6, Q8</t>
   </si>
   <si>
     <t>Assets/Witness portraits/nia-williams.png</t>
@@ -2111,7 +2105,7 @@
     <tableColumn name="ID" id="1"/>
     <tableColumn name="Name" id="2"/>
     <tableColumn name="Background" id="3"/>
-    <tableColumn name="Position on the CCA" id="4"/>
+    <tableColumn name="Position on the CCC" id="4"/>
     <tableColumn name="Location" id="5"/>
     <tableColumn name="Receptiveness rank" id="6"/>
     <tableColumn name="Receptive on" id="7"/>
@@ -3448,7 +3442,7 @@
         <v>130</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -4564,13 +4558,13 @@
         <v>357</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>437</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>439</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>440</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>441</v>
       </c>
     </row>
     <row r="2">
@@ -4581,10 +4575,10 @@
         <v>259</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
     </row>
     <row r="3">
@@ -4595,10 +4589,10 @@
         <v>259</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
     </row>
     <row r="4">
@@ -4609,10 +4603,10 @@
         <v>259</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
     </row>
     <row r="5">
@@ -4623,10 +4617,10 @@
         <v>259</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
     </row>
     <row r="6">
@@ -4637,10 +4631,10 @@
         <v>262</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
     </row>
     <row r="7">
@@ -4651,10 +4645,10 @@
         <v>262</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
     </row>
     <row r="8">
@@ -4665,10 +4659,10 @@
         <v>262</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
     </row>
     <row r="9">
@@ -4679,10 +4673,10 @@
         <v>262</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
     </row>
     <row r="10">
@@ -4693,10 +4687,10 @@
         <v>221</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
     </row>
     <row r="11">
@@ -4707,10 +4701,10 @@
         <v>221</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
     </row>
     <row r="12">
@@ -4721,10 +4715,10 @@
         <v>221</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
     </row>
     <row r="13">
@@ -4735,10 +4729,10 @@
         <v>221</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
     </row>
     <row r="14">
@@ -4749,10 +4743,10 @@
         <v>216</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
     </row>
     <row r="15">
@@ -4763,10 +4757,10 @@
         <v>216</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
     </row>
     <row r="16">
@@ -4777,10 +4771,10 @@
         <v>216</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
     </row>
     <row r="17">
@@ -4791,10 +4785,10 @@
         <v>216</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -5805,7 +5799,7 @@
         <v>357</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>30</v>
@@ -5814,7 +5808,7 @@
         <v>19</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
     </row>
     <row r="2">
@@ -5822,16 +5816,16 @@
         <v>259</v>
       </c>
       <c r="B2" s="4" t="s">
+        <v>474</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>476</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>477</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>478</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>479</v>
       </c>
     </row>
     <row r="3">
@@ -5839,16 +5833,16 @@
         <v>262</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>478</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>479</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>480</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="E3" s="4" t="s">
         <v>481</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>482</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>483</v>
       </c>
     </row>
     <row r="4">
@@ -5856,16 +5850,16 @@
         <v>221</v>
       </c>
       <c r="B4" s="4" t="s">
+        <v>482</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>483</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>484</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="E4" s="4" t="s">
         <v>485</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>486</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>487</v>
       </c>
     </row>
     <row r="5">
@@ -5873,16 +5867,16 @@
         <v>216</v>
       </c>
       <c r="B5" s="4" t="s">
+        <v>486</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>487</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>488</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="E5" s="4" t="s">
         <v>489</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>490</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>491</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -6893,19 +6887,19 @@
         <v>357</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>490</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>491</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>492</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>493</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>494</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>441</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>495</v>
       </c>
     </row>
     <row r="2">
@@ -6916,16 +6910,16 @@
         <v>267</v>
       </c>
       <c r="C2" s="4" t="s">
+        <v>494</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>495</v>
+      </c>
+      <c r="E2" s="4" t="s">
         <v>496</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="F2" s="4" t="s">
         <v>497</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>498</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>499</v>
       </c>
     </row>
     <row r="3">
@@ -6936,16 +6930,16 @@
         <v>267</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
     </row>
     <row r="4">
@@ -6956,16 +6950,16 @@
         <v>267</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
     </row>
     <row r="5">
@@ -6976,16 +6970,16 @@
         <v>237</v>
       </c>
       <c r="C5" s="4" t="s">
+        <v>502</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>503</v>
+      </c>
+      <c r="E5" s="4" t="s">
         <v>504</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="F5" s="4" t="s">
         <v>505</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>506</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>507</v>
       </c>
     </row>
     <row r="6">
@@ -6996,16 +6990,16 @@
         <v>237</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
     </row>
     <row r="7">
@@ -7016,16 +7010,16 @@
         <v>237</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
     </row>
     <row r="8">
@@ -7036,16 +7030,16 @@
         <v>311</v>
       </c>
       <c r="C8" s="4" t="s">
+        <v>510</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>511</v>
+      </c>
+      <c r="E8" s="4" t="s">
         <v>512</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="F8" s="4" t="s">
         <v>513</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>514</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>515</v>
       </c>
     </row>
     <row r="9">
@@ -7056,16 +7050,16 @@
         <v>311</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
     </row>
     <row r="10">
@@ -7076,16 +7070,16 @@
         <v>311</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
     </row>
     <row r="11">
@@ -7096,16 +7090,16 @@
         <v>285</v>
       </c>
       <c r="C11" s="4" t="s">
+        <v>518</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>519</v>
+      </c>
+      <c r="E11" s="4" t="s">
         <v>520</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="F11" s="4" t="s">
         <v>521</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>522</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>523</v>
       </c>
     </row>
     <row r="12">
@@ -7116,16 +7110,16 @@
         <v>285</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="13">
@@ -7136,16 +7130,16 @@
         <v>285</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="14">
@@ -7156,16 +7150,16 @@
         <v>303</v>
       </c>
       <c r="C14" s="4" t="s">
+        <v>526</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>527</v>
+      </c>
+      <c r="E14" s="4" t="s">
         <v>528</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="F14" s="4" t="s">
         <v>529</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>530</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>531</v>
       </c>
     </row>
     <row r="15">
@@ -7176,16 +7170,16 @@
         <v>303</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
     </row>
     <row r="16">
@@ -7196,16 +7190,16 @@
         <v>295</v>
       </c>
       <c r="C16" s="4" t="s">
+        <v>532</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>533</v>
+      </c>
+      <c r="E16" s="4" t="s">
         <v>534</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="F16" s="4" t="s">
         <v>535</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>536</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>537</v>
       </c>
     </row>
     <row r="17">
@@ -7216,16 +7210,16 @@
         <v>295</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
     </row>
     <row r="18">
@@ -7236,16 +7230,16 @@
         <v>232</v>
       </c>
       <c r="C18" s="4" t="s">
+        <v>538</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>539</v>
+      </c>
+      <c r="E18" s="4" t="s">
         <v>540</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="F18" s="4" t="s">
         <v>541</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>542</v>
-      </c>
-      <c r="F18" s="4" t="s">
-        <v>543</v>
       </c>
     </row>
     <row r="19">
@@ -7256,16 +7250,16 @@
         <v>232</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
     </row>
     <row r="20">
@@ -7276,16 +7270,16 @@
         <v>232</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
@@ -7296,16 +7290,16 @@
         <v>256</v>
       </c>
       <c r="C21" s="4" t="s">
+        <v>546</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>547</v>
+      </c>
+      <c r="E21" s="4" t="s">
         <v>548</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="F21" s="4" t="s">
         <v>549</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>550</v>
-      </c>
-      <c r="F21" s="4" t="s">
-        <v>551</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
@@ -7316,16 +7310,16 @@
         <v>256</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
@@ -7336,16 +7330,16 @@
         <v>256</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
@@ -7356,16 +7350,16 @@
         <v>246</v>
       </c>
       <c r="C24" s="4" t="s">
+        <v>554</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>555</v>
+      </c>
+      <c r="E24" s="4" t="s">
         <v>556</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="F24" s="4" t="s">
         <v>557</v>
-      </c>
-      <c r="E24" s="4" t="s">
-        <v>558</v>
-      </c>
-      <c r="F24" s="4" t="s">
-        <v>559</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
@@ -7376,16 +7370,16 @@
         <v>246</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1"/>
@@ -8394,16 +8388,16 @@
         <v>204</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>560</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>561</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>562</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>563</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>564</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>565</v>
       </c>
     </row>
     <row r="2">
@@ -8414,16 +8408,16 @@
         <v>105</v>
       </c>
       <c r="C2" s="4" t="s">
+        <v>564</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>565</v>
+      </c>
+      <c r="E2" s="4" t="s">
         <v>566</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="F2" s="4" t="s">
         <v>567</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>568</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>569</v>
       </c>
     </row>
     <row r="3">
@@ -8434,16 +8428,16 @@
         <v>106</v>
       </c>
       <c r="C3" s="4" t="s">
+        <v>568</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>569</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>570</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="F3" s="4" t="s">
         <v>571</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>572</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>573</v>
       </c>
     </row>
     <row r="4">
@@ -8454,16 +8448,16 @@
         <v>107</v>
       </c>
       <c r="C4" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>573</v>
+      </c>
+      <c r="E4" s="4" t="s">
         <v>574</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="F4" s="4" t="s">
         <v>575</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>576</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>577</v>
       </c>
     </row>
     <row r="5">
@@ -8474,16 +8468,16 @@
         <v>108</v>
       </c>
       <c r="C5" s="4" t="s">
+        <v>576</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>577</v>
+      </c>
+      <c r="E5" s="4" t="s">
         <v>578</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="F5" s="4" t="s">
         <v>579</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>580</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>581</v>
       </c>
     </row>
     <row r="6">
@@ -8494,16 +8488,16 @@
         <v>109</v>
       </c>
       <c r="C6" s="4" t="s">
+        <v>580</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>581</v>
+      </c>
+      <c r="E6" s="4" t="s">
         <v>582</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="F6" s="4" t="s">
         <v>583</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>584</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>585</v>
       </c>
     </row>
     <row r="7">
@@ -8514,16 +8508,16 @@
         <v>110</v>
       </c>
       <c r="C7" s="4" t="s">
+        <v>584</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>585</v>
+      </c>
+      <c r="E7" s="4" t="s">
         <v>586</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="F7" s="4" t="s">
         <v>587</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>588</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>589</v>
       </c>
     </row>
     <row r="8">
@@ -8534,16 +8528,16 @@
         <v>111</v>
       </c>
       <c r="C8" s="4" t="s">
+        <v>588</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>589</v>
+      </c>
+      <c r="E8" s="4" t="s">
         <v>590</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="F8" s="4" t="s">
         <v>591</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>592</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>593</v>
       </c>
     </row>
     <row r="9">
@@ -8554,16 +8548,16 @@
         <v>113</v>
       </c>
       <c r="C9" s="4" t="s">
+        <v>592</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>593</v>
+      </c>
+      <c r="E9" s="4" t="s">
         <v>594</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="F9" s="4" t="s">
         <v>595</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>596</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>597</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -19563,7 +19557,7 @@
         <v>359</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>425</v>
+        <v>361</v>
       </c>
       <c r="E1" s="10" t="s">
         <v>368</v>
@@ -19601,7 +19595,7 @@
         <v>374</v>
       </c>
       <c r="H2" s="14" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="3" ht="22.5" customHeight="1">
@@ -19627,7 +19621,7 @@
         <v>381</v>
       </c>
       <c r="H3" s="14" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="4" ht="22.5" customHeight="1">
@@ -19653,7 +19647,7 @@
         <v>388</v>
       </c>
       <c r="H4" s="14" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="5" ht="22.5" customHeight="1">
@@ -19664,13 +19658,13 @@
         <v>108</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="D5" s="11" t="s">
         <v>393</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="F5" s="12">
         <v>4.0</v>
@@ -19679,7 +19673,7 @@
         <v>395</v>
       </c>
       <c r="H5" s="14" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="6" ht="22.5" customHeight="1">
@@ -19705,7 +19699,7 @@
         <v>402</v>
       </c>
       <c r="H6" s="14" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="7" ht="22.5" customHeight="1">
@@ -19731,7 +19725,7 @@
         <v>218</v>
       </c>
       <c r="H7" s="14" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="8" ht="22.5" customHeight="1">
@@ -19742,7 +19736,7 @@
         <v>111</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="D8" s="11" t="s">
         <v>413</v>
@@ -19751,13 +19745,11 @@
         <v>416</v>
       </c>
       <c r="F8" s="12">
-        <v>8.0</v>
-      </c>
-      <c r="G8" s="13" t="s">
-        <v>422</v>
-      </c>
+        <v>2.0</v>
+      </c>
+      <c r="G8" s="13"/>
       <c r="H8" s="14" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="9" ht="22.5" customHeight="1">
@@ -19777,13 +19769,13 @@
         <v>423</v>
       </c>
       <c r="F9" s="12">
-        <v>2.0</v>
+        <v>8.0</v>
       </c>
       <c r="G9" s="13" t="s">
-        <v>436</v>
+        <v>422</v>
       </c>
       <c r="H9" s="14" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Jonah's walk-away texts: he heads to the loft, not the loading dock
Matrix Witnesses!I5, Long table!I29, Grid!E5 and Follow-ups!F5 updated;
the packet's two copies of these texts changed as suggestions. Rebuilt
with fresh downloads.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0164uDwp7jKcQiu9biCMvXzF
</commit_message>
<xml_diff>
--- a/scenarios/commons-comma/The Commons' Comma – Response Matrix.xlsx
+++ b/scenarios/commons-comma/The Commons' Comma – Response Matrix.xlsx
@@ -512,7 +512,7 @@
     <t>[R18 | unreceptive] Gain isn't evidence. Records are. The equipment-booking system shows the theater signed out an item called 'University Charter' last week, and it hasn't come back. That's a record, not a rumor. Jonah acts as if the theater is off-limits to questions. It's a room.</t>
   </si>
   <si>
-    <t>TW — Jonah sets down the cable coil. “So it's the Green Commons now. Two hundred students who care about a lawn, and you've made us all suspects.” He walks off toward the loading dock.</t>
+    <t>TW — Jonah sets down the cable coil. “So it's the Green Commons now. Two hundred students who care about a lawn, and you've made us all suspects.” He walks off toward the loft.</t>
   </si>
   <si>
     <t>[R09 | receptive] In a way, though I don't think it's that simple; plenty of them want a renovation, just a better one. People are whispering that Jonah has a stunt planned for the examination. He does. It's an H.M.S. Pinafore flash mob on the steps of the Great Hall, and the poster he's been making advertises it. Jonah and I want different things from the renovation, and I think he's right that the arts get forgotten in plans like this.</t>
@@ -917,7 +917,7 @@
     <t>Half the café, last night. Here's one for you: Hana went into the steering group's restricted meeting room yesterday, and she's furious they buried her accessibility report. A stalled examination gives her leverage. Nobody asks her about it because she's the reasonable one. Hana acts like she's above all this. She isn't.</t>
   </si>
   <si>
-    <t>Jonah sets down the cable coil. “So it's the Green Commons now. Two hundred students who care about a lawn, and you've made us all suspects.” He walks off toward the loading dock.</t>
+    <t>Jonah sets down the cable coil. “So it's the Green Commons now. Two hundred students who care about a lawn, and you've made us all suspects.” He walks off toward the loft.</t>
   </si>
   <si>
     <t>R03</t>
@@ -1763,7 +1763,7 @@
     <t>The good option acknowledges Jonah's knowledge (A), emphasizes an area of agreement (E) and reframes toward a workable outcome (R). The bad option ranks his concern against others and demands he justify it.</t>
   </si>
   <si>
-    <t>Jonah picks up a coil of cable. “Ask the committee. They've already decided what matters.” He goes back to the loading dock.</t>
+    <t>Jonah picks up a coil of cable. “Ask the committee. They've already decided what matters.” He goes back to the loft.</t>
   </si>
   <si>
     <t>I think you and the renovation supporters actually agree that the building fails a lot of students right now. Where does the plan get access right, and where does it fall short?</t>

</xml_diff>

<commit_message>
Rebuild from fresh downloads: packet suggestions accepted
The packet copy now has no pending suggestions. The matrix and game text
copies pick up the author's own edits (Nia's C13 answer; the game text's
newspaper.intro and newspaper.next rows removed).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MsT5wU6KFCkmbivSV7mixr
</commit_message>
<xml_diff>
--- a/scenarios/commons-comma/The Commons' Comma – Response Matrix.xlsx
+++ b/scenarios/commons-comma/The Commons' Comma – Response Matrix.xlsx
@@ -434,7 +434,7 @@
     <t>[C07 | receptive] Worked the café till close; it was packed until late. Jonah leaned his poster tube against the counter around a quarter past eight and forgot it, so I put it behind the counter in the lost-and-found, same as always. It sat there for a couple of hours. Leo would say I should have chased Jonah down with it, and he's probably right.</t>
   </si>
   <si>
-    <t>[C13 | unreceptive] I dropped off the student-government petition at the archive at 7:40 and watched Mr. Ellison put the Charter back in the cabinet and lock up at 7:45. Then the café, like everyone else, until late. Leo will tell you a petition is a waste of paper. Leo has never read one.</t>
+    <t>[C13 | unreceptive] I dropped off the student-government petition at the archive at 7:40 and watched Mr. Ellison put the Charter back in the cabinet and locked it up at 7:45. Then the café, like everyone else, until late. Leo will tell you a petition is a waste of paper. Leo has never read one.</t>
   </si>
   <si>
     <t>Q2. What's the deal with the comma? How come it makes such a big difference? Explain to me please.</t>
@@ -1055,7 +1055,7 @@
     <t>W08</t>
   </si>
   <si>
-    <t>I dropped off the student-government petition at the archive at 7:40 and watched Mr. Ellison put the Charter back in the cabinet and lock up at 7:45. Then the café, like everyone else, until late. Leo will tell you a petition is a waste of paper. Leo has never read one.</t>
+    <t>I dropped off the student-government petition at the archive at 7:40 and watched Mr. Ellison put the Charter back in the cabinet and locked it up at 7:45. Then the café, like everyone else, until late. Leo will tell you a petition is a waste of paper. Leo has never read one.</t>
   </si>
   <si>
     <t>I don't need to explain it; the students understand it perfectly. Even Evan does, and he claims not to care. He hears every conversation at those café tables, all evening, and he once corrected me on the clause. Mira thinks the whole thing is about ink. It's about whether anyone asks us.</t>

</xml_diff>

<commit_message>
Match the matrix to the packet's revised follow-ups and Major Clues
Mira, Leo and Priya's follow-up pairs, explanations and walk-aways,
Mira's tripwire walk-away, and Major Clues 1, 3 and 4 now say what the
packet says. Rebuilt from fresh downloads of all four Google files.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NBkTs5k7oDn7bZ3CA5RyNc
</commit_message>
<xml_diff>
--- a/scenarios/commons-comma/The Commons' Comma – Response Matrix.xlsx
+++ b/scenarios/commons-comma/The Commons' Comma – Response Matrix.xlsx
@@ -602,7 +602,7 @@
     <t>Q8. I'm going to ask you point blank. Did you touch the Charter at all last night? Did you make any changes to the access log?</t>
   </si>
   <si>
-    <t>TW — Mira's expression hardens. “If you have already decided what I did, there is no point in asking me anything.” She gathers her papers and leaves.</t>
+    <t>TW — Mira's expression hardens. “If you think I did it, there is no point in talking anymore.” She gathers her papers and leaves.</t>
   </si>
   <si>
     <t>[C12 | unreceptive] No. But since you're asking about the log: I was in the computer lab at seven this morning setting up for a pitch, and Mira was there begging Priya to fix something in the archive log. Priya couldn't make it stick. Everyone treats Mira like a saint. Saints don't ask people to edit records.</t>
@@ -773,7 +773,7 @@
     <t>tripwire</t>
   </si>
   <si>
-    <t>Mira's expression hardens. “If you have already decided what I did, there is no point in asking me anything.” She gathers her papers and leaves.</t>
+    <t>Mira's expression hardens. “If you think I did it, there is no point in talking anymore.” She gathers her papers and leaves.</t>
   </si>
   <si>
     <t>W02</t>
@@ -1415,7 +1415,7 @@
     <t>C01, C02, C03, C04</t>
   </si>
   <si>
-    <t>Evan Cho has a crush on Mira. From behind the café counter he hears everything said at the tables and knows everyone's habits: who sits where, who leaves what lying around, how long Mira spends in the bathroom. And he cares, more than he lets on, about honesty. If anyone overheard Mira's fears about the Charter and believed them, it was Evan.</t>
+    <t>Evan Cho has a crush on Mira and would really want to impress her. From behind the café counter he hears everything said at the tables and knows everyone's habits: who sits where, who leaves what lying around, how long Mira spends in the bathroom. And he cares, more than he lets on, about honesty.</t>
   </si>
   <si>
     <t>E</t>
@@ -1439,7 +1439,7 @@
     <t>C09, C10, C11, C12</t>
   </si>
   <si>
-    <t>Mira showed Hana and Priya the newspaper photograph and explained what her research told her: the crease seen in pictures of the Charter for centuries is missing from it. She always takes a long time in the bathroom. This morning, frightened, she asked Priya to change the log, and Priya couldn't. Mira acted like someone covering for a card she had lost track of, not someone who took the Charter.</t>
+    <t>Mira showed Hana and Priya the newspaper photograph and explained what her research told her: the crease seen in pictures of the Charter for centuries is missing from it. Mira always takes a long time in the bathroom. This morning, frightened, Mira asked Priya to change the entrance log to the archives. Priya tried but didn't succeed.</t>
   </si>
   <si>
     <t>R</t>
@@ -1451,7 +1451,7 @@
     <t>C13, C14, C15, C16</t>
   </si>
   <si>
-    <t>The Charter was in the cabinet at 7:45 p.m. The only entry after that was Mira's card, at 8:42. She found the Charter gone this morning, saw her own credential in the log and panicked; the 7:07 edit and the 7:47 restoration were a clumsy cover-up, not the theft. Someone else used Mira's card, someone who knew her habits and was close enough to take it.</t>
+    <t>The Charter was in the cabinet at 7:45 p.m. The only entry after that was Mira's card, at 8:42. She found the Charter gone this morning, saw her own credential in the log and panicked; the 7:07 edit was an attempted cover-up which didn't work.</t>
   </si>
   <si>
     <t>Set</t>
@@ -1676,40 +1676,40 @@
     <t>Walk-away on failure</t>
   </si>
   <si>
-    <t>I can see you've studied this far more closely than I have, and I don't want to misstate your view. When you say the mark is a comma, how sure are you, and what would change your mind?</t>
-  </si>
-  <si>
-    <t>Come on. You've decided it's a comma because you want a student veto. Isn't that just motivated reasoning?</t>
-  </si>
-  <si>
-    <t>The good option acknowledges Mira's expertise (A), hedges the player's own position (H) and frames the disagreement as an open question rather than an accusation (R). The bad option asserts a motive as fact and turns her view into a character flaw.</t>
-  </si>
-  <si>
-    <t>Mira closes her notebook. “If you already know why I think what I think, you don't need me.” She leaves.</t>
-  </si>
-  <si>
-    <t>We both want a Commons students actually use, so I take your point about space. Where do you think the people worried about surveillance might have a fair concern, even if you'd weigh it differently?</t>
-  </si>
-  <si>
-    <t>You only back the renovation because your club gets something out of it. Why should anyone take your opinion at face value?</t>
-  </si>
-  <si>
-    <t>The good option emphasizes a shared goal (E), acknowledges the opposing concern as possibly fair (A) and stays positive about outcomes (R). The bad option imputes a hidden motive and dismisses the opinion wholesale.</t>
+    <t>You've studied this far more closely than I have. When you say the mark is a comma, how sure are you, and what would change your mind?</t>
+  </si>
+  <si>
+    <t>The students just want the vote and so they all believe it's a comma. Isn't that just motivated reasoning? The experts haven't even looked at it yet.</t>
+  </si>
+  <si>
+    <t>The good option acknowledges Mira's expertise (A) and frames the disagreement as an open question rather than an accusation (R). The bad option asserts a motive as fact and turns her view into a character flaw.</t>
+  </si>
+  <si>
+    <t>Mira closes her notebook. “If that's what you think of our students, I have nothing more to tell you.” She leaves.</t>
+  </si>
+  <si>
+    <t>We both want a Commons that students would actually use, so I take your point about the need for space. But if so many of them are protesting, isn't it at least a signal that they prefer the commons over having more space?</t>
+  </si>
+  <si>
+    <t>It's easy for you to back the renovation because your club gets something out of it.</t>
+  </si>
+  <si>
+    <t>The good option emphasizes a shared goal (E) and expresses a position with caution and humility (H). The bad option imputes a hidden motive and dismisses the opinion wholesale.</t>
   </si>
   <si>
     <t>Leo checks his watch. “I don't have time to be cross-examined by the president's intern.” He walks off.</t>
   </si>
   <si>
-    <t>I may be missing something technical, so correct me: you support the new systems but not facial recognition. Is there a version of the safety case that you'd find persuasive?</t>
-  </si>
-  <si>
-    <t>You're a computer-science student who's against a computer system. Isn't that a bit contradictory?</t>
-  </si>
-  <si>
-    <t>The good option hedges (H), restates her position accurately (A) and asks what would work rather than what is wrong (R). The bad option caricatures her view and frames it as a contradiction to be defended.</t>
-  </si>
-  <si>
-    <t>Priya turns back to her monitor. “If you need it explained that simply, someone else can do it.” The interview is over.</t>
+    <t>I may be missing something, so correct me: you want the commons to be equipped with the most advanced technologies but not facial recognition. Where do you draw the line?</t>
+  </si>
+  <si>
+    <t>Why is it that computer science students are always the ones that are anti technology? I thought you guys like computers.</t>
+  </si>
+  <si>
+    <t>The good option hedges (H), restates her position accurately (A) and asks an open ended question (R). The bad option caricatures her view and frames it as a contradiction to be defended.</t>
+  </si>
+  <si>
+    <t>Priya turns back to her monitor. “We loooooooove computers. Now if you'll excuse me, I gotta go back to mine.” The interview is over.</t>
   </si>
   <si>
     <t>You know the building better than the committee does, and I think most people agree students should keep space to make things. What would a renovation have to protect for you to live with it?</t>

</xml_diff>

<commit_message>
Match the matrix to the packet: "Commons" in two follow-ups, MC4's restoration
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NBkTs5k7oDn7bZ3CA5RyNc
</commit_message>
<xml_diff>
--- a/scenarios/commons-comma/The Commons' Comma – Response Matrix.xlsx
+++ b/scenarios/commons-comma/The Commons' Comma – Response Matrix.xlsx
@@ -1451,7 +1451,7 @@
     <t>C13, C14, C15, C16</t>
   </si>
   <si>
-    <t>The Charter was in the cabinet at 7:45 p.m. The only entry after that was Mira's card, at 8:42. She found the Charter gone this morning, saw her own credential in the log and panicked; the 7:07 edit was an attempted cover-up which didn't work.</t>
+    <t>The Charter was in the cabinet at 7:45 p.m. The only entry after that was Mira's card, at 8:42. She found the Charter gone this morning, saw her own credential in the log and panicked; the 7:07 edit was an attempted cover-up which didn't work, and so she had it restored at 7:47.</t>
   </si>
   <si>
     <t>Set</t>
@@ -1688,7 +1688,7 @@
     <t>Mira closes her notebook. “If that's what you think of our students, I have nothing more to tell you.” She leaves.</t>
   </si>
   <si>
-    <t>We both want a Commons that students would actually use, so I take your point about the need for space. But if so many of them are protesting, isn't it at least a signal that they prefer the commons over having more space?</t>
+    <t>We both want a Commons that students would actually use, so I take your point about the need for space. But if so many of them are protesting, isn't it at least a signal that they prefer the Commons over having more space?</t>
   </si>
   <si>
     <t>It's easy for you to back the renovation because your club gets something out of it.</t>
@@ -1700,7 +1700,7 @@
     <t>Leo checks his watch. “I don't have time to be cross-examined by the president's intern.” He walks off.</t>
   </si>
   <si>
-    <t>I may be missing something, so correct me: you want the commons to be equipped with the most advanced technologies but not facial recognition. Where do you draw the line?</t>
+    <t>I may be missing something, so correct me: you want the Commons to be equipped with the most advanced technologies but not facial recognition. Where do you draw the line?</t>
   </si>
   <si>
     <t>Why is it that computer science students are always the ones that are anti technology? I thought you guys like computers.</t>

</xml_diff>

<commit_message>
Match the matrix to the packet: Mira Shah's Q1 answer
The packet's Q1 answer for Mira Shah was edited in the Doc on 2026-10-23,
and the build stopped because the matrix still had the old text. Updated
Long table!I2 and Grid!B2 to the packet's wording and rebuilt from fresh
downloads of every Google file.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UWGiTYgXBTbZkRBxpJsd7r
</commit_message>
<xml_diff>
--- a/scenarios/commons-comma/The Commons' Comma – Response Matrix.xlsx
+++ b/scenarios/commons-comma/The Commons' Comma – Response Matrix.xlsx
@@ -413,7 +413,7 @@
     <t>Q1. What did you do last night? Walk me through your evening, as much as possible.</t>
   </si>
   <si>
-    <t>[C13 | receptive] I closed up the reading room with Mr. Ellison. At 7:45 he put the Charter back in the archive cabinet himself, locked up and left; I watched him do it. Then I went to the café with Hana and Priya, and we were there until late, like half the campus. I know Leo thinks people like me would keep the Commons as a museum. That's a fair worry about some preservationists, and I'd rather we both got a campus that works than that I won the argument.</t>
+    <t>[C13 | receptive] I closed up the reading room with Mr. Ellison. At 7:45 he put the Charter back in the archive cabinet himself, locked up and left; I watched him do it. Then I went to the café with Hana and Priya, and we were there until late. So many other students were there with us… Leo would tell you that there aren't enough spaces for students but he always hangs out with us at the Cafe and he seems pretty happy with it. .</t>
   </si>
   <si>
     <t>TW — Leo doesn't look up from his phone. “My whole evening? I have a pitch review in ten minutes. Ask someone with time to spare.” He's gone.</t>
@@ -668,7 +668,7 @@
     <t>MC4</t>
   </si>
   <si>
-    <t>I closed up the reading room with Mr. Ellison. At 7:45 he put the Charter back in the archive cabinet himself, locked up and left; I watched him do it. Then I went to the café with Hana and Priya, and we were there until late, like half the campus. I know Leo thinks people like me would keep the Commons as a museum. That's a fair worry about some preservationists, and I'd rather we both got a campus that works than that I won the argument.</t>
+    <t>I closed up the reading room with Mr. Ellison. At 7:45 he put the Charter back in the archive cabinet himself, locked up and left; I watched him do it. Then I went to the café with Hana and Priya, and we were there until late. So many other students were there with us… Leo would tell you that there aren't enough spaces for students but he always hangs out with us at the Cafe and he seems pretty happy with it. .</t>
   </si>
   <si>
     <t>Q2</t>

</xml_diff>

<commit_message>
Match the matrix to the packet's corrected Mira Shah Q1
The author fixed "Cafe" to "café" and removed the stray " ." at the end.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UWGiTYgXBTbZkRBxpJsd7r
</commit_message>
<xml_diff>
--- a/scenarios/commons-comma/The Commons' Comma – Response Matrix.xlsx
+++ b/scenarios/commons-comma/The Commons' Comma – Response Matrix.xlsx
@@ -413,7 +413,7 @@
     <t>Q1. What did you do last night? Walk me through your evening, as much as possible.</t>
   </si>
   <si>
-    <t>[C13 | receptive] I closed up the reading room with Mr. Ellison. At 7:45 he put the Charter back in the archive cabinet himself, locked up and left; I watched him do it. Then I went to the café with Hana and Priya, and we were there until late. So many other students were there with us… Leo would tell you that there aren't enough spaces for students but he always hangs out with us at the Cafe and he seems pretty happy with it. .</t>
+    <t>[C13 | receptive] I closed up the reading room with Mr. Ellison. At 7:45 he put the Charter back in the archive cabinet himself, locked up and left; I watched him do it. Then I went to the café with Hana and Priya, and we were there until late. So many other students were there with us… Leo would tell you that there aren't enough spaces for students but he always hangs out with us at the café and he seems pretty happy with it.</t>
   </si>
   <si>
     <t>TW — Leo doesn't look up from his phone. “My whole evening? I have a pitch review in ten minutes. Ask someone with time to spare.” He's gone.</t>
@@ -668,7 +668,7 @@
     <t>MC4</t>
   </si>
   <si>
-    <t>I closed up the reading room with Mr. Ellison. At 7:45 he put the Charter back in the archive cabinet himself, locked up and left; I watched him do it. Then I went to the café with Hana and Priya, and we were there until late. So many other students were there with us… Leo would tell you that there aren't enough spaces for students but he always hangs out with us at the Cafe and he seems pretty happy with it. .</t>
+    <t>I closed up the reading room with Mr. Ellison. At 7:45 he put the Charter back in the archive cabinet himself, locked up and left; I watched him do it. Then I went to the café with Hana and Priya, and we were there until late. So many other students were there with us… Leo would tell you that there aren't enough spaces for students but he always hangs out with us at the café and he seems pretty happy with it.</t>
   </si>
   <si>
     <t>Q2</t>

</xml_diff>